<commit_message>
add data from daily run
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -600,6 +600,44 @@
         <v>4</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>20522</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="n">
+        <v>304.925827717781</v>
+      </c>
+      <c r="E4" t="n">
+        <v>67</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>590</v>
+      </c>
+      <c r="H4" t="n">
+        <v>104</v>
+      </c>
+      <c r="I4" t="n">
+        <v>486</v>
+      </c>
+      <c r="J4" t="n">
+        <v>35</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1043</v>
+      </c>
+      <c r="L4" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
adding data from daily run
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -638,6 +638,44 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>20523</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" t="n">
+        <v>197.715229813258</v>
+      </c>
+      <c r="E5" t="n">
+        <v>72</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>623</v>
+      </c>
+      <c r="H5" t="n">
+        <v>98</v>
+      </c>
+      <c r="I5" t="n">
+        <v>525</v>
+      </c>
+      <c r="J5" t="n">
+        <v>17</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1218</v>
+      </c>
+      <c r="L5" t="n">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
add data from new run
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -676,6 +676,44 @@
         <v>8</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>20524</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" t="n">
+        <v>225.004321316878</v>
+      </c>
+      <c r="E6" t="n">
+        <v>76</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>669</v>
+      </c>
+      <c r="H6" t="n">
+        <v>104</v>
+      </c>
+      <c r="I6" t="n">
+        <v>565</v>
+      </c>
+      <c r="J6" t="n">
+        <v>27</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1279</v>
+      </c>
+      <c r="L6" t="n">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
adding data from new run
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -714,6 +714,44 @@
         <v>6</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>20525</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="n">
+        <v>213.896635647615</v>
+      </c>
+      <c r="E7" t="n">
+        <v>75</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>687</v>
+      </c>
+      <c r="H7" t="n">
+        <v>81</v>
+      </c>
+      <c r="I7" t="n">
+        <v>606</v>
+      </c>
+      <c r="J7" t="n">
+        <v>19</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1315</v>
+      </c>
+      <c r="L7" t="n">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
adding data from daily run"
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -1474,6 +1474,44 @@
         <v>8</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>20547</v>
+      </c>
+      <c r="B27" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" t="s">
+        <v>27</v>
+      </c>
+      <c r="D27" t="n">
+        <v>297.225667369366</v>
+      </c>
+      <c r="E27" t="n">
+        <v>95</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="n">
+        <v>767</v>
+      </c>
+      <c r="H27" t="n">
+        <v>130</v>
+      </c>
+      <c r="I27" t="n">
+        <v>637</v>
+      </c>
+      <c r="J27" t="n">
+        <v>123</v>
+      </c>
+      <c r="K27" t="n">
+        <v>3211</v>
+      </c>
+      <c r="L27" t="n">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update scraped data [2026-04-24]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
   <si>
     <t>date</t>
   </si>
@@ -126,6 +126,12 @@
   </si>
   <si>
     <t xml:space="preserve">final_score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f74fa3de3ad0c7973382d90fdaced59b8ed8ceec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/colombia/primera-a/, /football/el-salvador/primera-division/, /football/greece/super-league/, /football/guatemala/liga-nacional/, /football/netherlands/eredivisie/, /football/paraguay/division-intermedia/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -133,19 +139,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -173,10 +173,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -595,7 +594,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>20521</v>
       </c>
       <c r="B3"/>
@@ -634,7 +633,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>20522</v>
       </c>
       <c r="B4"/>
@@ -673,7 +672,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>20523</v>
       </c>
       <c r="B5"/>
@@ -712,7 +711,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>20524</v>
       </c>
       <c r="B6"/>
@@ -751,7 +750,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>20525</v>
       </c>
       <c r="B7"/>
@@ -790,7 +789,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>20526</v>
       </c>
       <c r="B8"/>
@@ -829,7 +828,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>20527</v>
       </c>
       <c r="B9"/>
@@ -868,7 +867,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>20528</v>
       </c>
       <c r="B10"/>
@@ -907,7 +906,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>20529</v>
       </c>
       <c r="B11"/>
@@ -946,7 +945,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>20530</v>
       </c>
       <c r="B12"/>
@@ -985,7 +984,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>20531</v>
       </c>
       <c r="B13"/>
@@ -1024,7 +1023,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="1" t="n">
         <v>20532</v>
       </c>
       <c r="B14"/>
@@ -1063,7 +1062,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="1" t="n">
         <v>20533</v>
       </c>
       <c r="B15"/>
@@ -1102,7 +1101,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="1" t="n">
         <v>20534</v>
       </c>
       <c r="B16"/>
@@ -1141,7 +1140,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="1" t="n">
         <v>20535</v>
       </c>
       <c r="B17"/>
@@ -1180,7 +1179,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="1" t="n">
         <v>20536</v>
       </c>
       <c r="B18"/>
@@ -1219,7 +1218,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="1" t="n">
         <v>20537</v>
       </c>
       <c r="B19"/>
@@ -1258,7 +1257,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="1" t="n">
         <v>20539</v>
       </c>
       <c r="B20"/>
@@ -1297,7 +1296,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="1" t="n">
         <v>20540</v>
       </c>
       <c r="B21"/>
@@ -1336,7 +1335,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="1" t="n">
         <v>20541</v>
       </c>
       <c r="B22"/>
@@ -1375,7 +1374,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="1" t="n">
         <v>20542</v>
       </c>
       <c r="B23"/>
@@ -1414,7 +1413,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="1" t="n">
         <v>20543</v>
       </c>
       <c r="B24"/>
@@ -1453,7 +1452,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="1" t="n">
         <v>20545</v>
       </c>
       <c r="B25"/>
@@ -1492,7 +1491,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="1" t="n">
         <v>20546</v>
       </c>
       <c r="B26"/>
@@ -1531,7 +1530,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="1" t="n">
         <v>20547</v>
       </c>
       <c r="B27"/>
@@ -1570,7 +1569,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="1" t="n">
         <v>20548</v>
       </c>
       <c r="B28"/>
@@ -1609,7 +1608,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="1" t="n">
         <v>20549</v>
       </c>
       <c r="B29"/>
@@ -1648,7 +1647,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="1" t="n">
         <v>20551</v>
       </c>
       <c r="B30"/>
@@ -1687,7 +1686,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="1" t="n">
         <v>20555</v>
       </c>
       <c r="B31"/>
@@ -1726,7 +1725,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="1" t="n">
         <v>20556</v>
       </c>
       <c r="B32"/>
@@ -1765,7 +1764,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="1" t="n">
         <v>20557</v>
       </c>
       <c r="B33"/>
@@ -1804,7 +1803,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="1" t="n">
         <v>20558</v>
       </c>
       <c r="B34"/>
@@ -1843,7 +1842,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="1" t="n">
         <v>20559</v>
       </c>
       <c r="B35"/>
@@ -1882,7 +1881,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="1" t="n">
         <v>20560</v>
       </c>
       <c r="B36"/>
@@ -1921,7 +1920,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="1" t="n">
         <v>20561</v>
       </c>
       <c r="B37"/>
@@ -1960,7 +1959,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="1" t="n">
         <v>20562</v>
       </c>
       <c r="B38"/>
@@ -1999,7 +1998,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="1" t="n">
         <v>20563</v>
       </c>
       <c r="B39"/>
@@ -2038,7 +2037,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="1" t="n">
         <v>46135</v>
       </c>
       <c r="B40" t="s">
@@ -2076,6 +2075,47 @@
       </c>
       <c r="M40" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B41" t="s">
+        <v>37</v>
+      </c>
+      <c r="C41" t="s">
+        <v>31</v>
+      </c>
+      <c r="D41" t="n">
+        <v>242.564734427134</v>
+      </c>
+      <c r="E41" t="n">
+        <v>70</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" t="n">
+        <v>500</v>
+      </c>
+      <c r="H41" t="n">
+        <v>75</v>
+      </c>
+      <c r="I41" t="n">
+        <v>425</v>
+      </c>
+      <c r="J41" t="n">
+        <v>24</v>
+      </c>
+      <c r="K41" t="n">
+        <v>3826</v>
+      </c>
+      <c r="L41" t="n">
+        <v>22</v>
+      </c>
+      <c r="M41" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update scraped data [2026-04-25]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
   <si>
     <t>date</t>
   </si>
@@ -138,6 +138,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/2-liga/, /football/greece/super-league/, /football/guatemala/liga-nacional/, /football/latvia/virsliga/, /football/netherlands/eredivisie/, /football/netherlands/eerste-divisie/, /football/panama/lpf/, /football/paraguay/division-intermedia/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e12601a9dd84076c73c95870a3d0d2e99ad53729</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/colombia/primera-a/, /football/greece/super-league/, /football/japan/j1-league/, /football/latvia/virsliga/, /football/netherlands/eredivisie/, /football/sierra-leone/premier-league/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -2165,6 +2171,47 @@
         <v>40</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B43" t="s">
+        <v>41</v>
+      </c>
+      <c r="C43" t="s">
+        <v>31</v>
+      </c>
+      <c r="D43" t="n">
+        <v>273.553482600053</v>
+      </c>
+      <c r="E43" t="n">
+        <v>80</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" t="n">
+        <v>498</v>
+      </c>
+      <c r="H43" t="n">
+        <v>85</v>
+      </c>
+      <c r="I43" t="n">
+        <v>413</v>
+      </c>
+      <c r="J43" t="n">
+        <v>54</v>
+      </c>
+      <c r="K43" t="n">
+        <v>4220</v>
+      </c>
+      <c r="L43" t="n">
+        <v>33</v>
+      </c>
+      <c r="M43" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-04-26]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="46">
   <si>
     <t>date</t>
   </si>
@@ -150,6 +150,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/ethiopia/premier-league/, /football/finland/veikkausliiga/, /football/greece/super-league/, /football/ireland/premier-division/, /football/netherlands/eredivisie/, /football/romania/superliga/, /football/uruguay/segunda-division/, /football/venezuela/liga-futve-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1001fdf0d6926a6133d9d392d4e8ec6604e24d36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/finland/veikkausliiga/, /football/greece/super-league/, /football/ireland/premier-division/, /football/ireland/division-1/, /football/latvia/virsliga/, /football/romania/superliga/, /football/south-korea/k-league-2/, /football/sweden/superettan/</t>
   </si>
 </sst>
 </file>
@@ -2259,6 +2265,47 @@
         <v>44</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B45" t="s">
+        <v>45</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45" t="n">
+        <v>209.198676315943</v>
+      </c>
+      <c r="E45" t="n">
+        <v>76</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>413</v>
+      </c>
+      <c r="H45" t="n">
+        <v>95</v>
+      </c>
+      <c r="I45" t="n">
+        <v>318</v>
+      </c>
+      <c r="J45" t="n">
+        <v>82</v>
+      </c>
+      <c r="K45" t="n">
+        <v>4143</v>
+      </c>
+      <c r="L45" t="n">
+        <v>32</v>
+      </c>
+      <c r="M45" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-04-27]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="50">
   <si>
     <t>date</t>
   </si>
@@ -162,6 +162,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/2-liga/, /football/denmark/1st-division/, /football/estonia/meistriliiga/, /football/ethiopia/premier-league/, /football/finland/veikkausliiga/, /football/finland/ykkosliiga/, /football/finland/ykkosliiga/, /football/iraq/stars-league/, /football/ireland/division-1/, /football/norway/obos-ligaen/, /football/peru/liga-1/, /football/poland/division-1/, /football/romania/superliga/, /football/romania/liga-2/, /football/slovenia/prva-liga/, /football/south-korea/k-league-2/, /football/turkey/1-lig/, /football/turkey/1-lig/, /football/ukraine/premier-league/, /football/venezuela/liga-futve-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4cd0587c2302deda576187a47654f862bdc5b60a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/croatia/hnl/, /football/denmark/1st-division/, /football/ireland/division-1/, /football/norway/obos-ligaen/, /football/romania/superliga/, /football/romania/liga-2/, /football/sweden/superettan/, /football/ukraine/premier-league/, /football/uzbekistan/super-league/</t>
   </si>
 </sst>
 </file>
@@ -2353,6 +2359,47 @@
         <v>48</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B47" t="s">
+        <v>49</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47" t="n">
+        <v>249.772590577602</v>
+      </c>
+      <c r="E47" t="n">
+        <v>59</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>364</v>
+      </c>
+      <c r="H47" t="n">
+        <v>112</v>
+      </c>
+      <c r="I47" t="n">
+        <v>252</v>
+      </c>
+      <c r="J47" t="n">
+        <v>47</v>
+      </c>
+      <c r="K47" t="n">
+        <v>3403</v>
+      </c>
+      <c r="L47" t="n">
+        <v>14</v>
+      </c>
+      <c r="M47" t="s">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-04-28]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="54">
   <si>
     <t>date</t>
   </si>
@@ -174,6 +174,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/croatia/hnl/, /football/denmark/1st-division/, /football/estonia/esiliiga/, /football/ireland/division-1/, /football/peru/liga-1/, /football/romania/superliga/, /football/romania/liga-2/, /football/slovenia/prva-liga/, /football/south-korea/k-league-2/, /football/turkey/1-lig/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">535fc9419b8af87d8be52de3973f2bb2a98447b5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/colombia/primera-b/, /football/ukraine/premier-league/, /football/uruguay/liga-auf-uruguaya/</t>
   </si>
 </sst>
 </file>
@@ -2447,6 +2453,47 @@
         <v>52</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B49" t="s">
+        <v>53</v>
+      </c>
+      <c r="C49" t="s">
+        <v>31</v>
+      </c>
+      <c r="D49" t="n">
+        <v>177.797466667493</v>
+      </c>
+      <c r="E49" t="n">
+        <v>51</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" t="n">
+        <v>370</v>
+      </c>
+      <c r="H49" t="n">
+        <v>69</v>
+      </c>
+      <c r="I49" t="n">
+        <v>301</v>
+      </c>
+      <c r="J49" t="n">
+        <v>27</v>
+      </c>
+      <c r="K49" t="n">
+        <v>3259</v>
+      </c>
+      <c r="L49" t="n">
+        <v>15</v>
+      </c>
+      <c r="M49" t="s">
+        <v>54</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-04-29]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="58">
   <si>
     <t>date</t>
   </si>
@@ -186,6 +186,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/chile/liga-de-ascenso/, /football/colombia/primera-b/, /football/ethiopia/premier-league/, /football/finland/ykkosliiga/, /football/honduras/liga-nacional/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/luxembourg/bgl-ligue/, /football/peru/liga-1/, /football/turkey/1-lig/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">980f7f0ce93dd88afe20f5bcbca467cbd45534f8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/cameroon/elite-one/, /football/china/super-league/, /football/estonia/esiliiga/, /football/japan/j1-league/, /football/lithuania/i-lyga/, /football/peru/liga-1/, /football/south-america/copa-sudamericana/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -2541,6 +2547,47 @@
         <v>56</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B51" t="s">
+        <v>57</v>
+      </c>
+      <c r="C51" t="s">
+        <v>31</v>
+      </c>
+      <c r="D51" t="n">
+        <v>247.283576309681</v>
+      </c>
+      <c r="E51" t="n">
+        <v>57</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" t="n">
+        <v>404</v>
+      </c>
+      <c r="H51" t="n">
+        <v>116</v>
+      </c>
+      <c r="I51" t="n">
+        <v>288</v>
+      </c>
+      <c r="J51" t="n">
+        <v>19</v>
+      </c>
+      <c r="K51" t="n">
+        <v>3786</v>
+      </c>
+      <c r="L51" t="n">
+        <v>19</v>
+      </c>
+      <c r="M51" t="s">
+        <v>58</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-04-30]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
   <si>
     <t>date</t>
   </si>
@@ -198,6 +198,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/colombia/primera-a/, /football/colombia/primera-b/, /football/ethiopia/premier-league/, /football/faroe-islands/premier-league/, /football/finland/ykkosliiga/, /football/iceland/division-1/, /football/ireland/division-1/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/lithuania/i-lyga/, /football/peru/liga-1/, /football/turkey/1-lig/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eb7e4c010c29a12293d4228b76893a9de75a1a59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/finland/ykkosliiga/, /football/georgia/crystalbet-erovnuli-liga/, /football/turkey/1-lig/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -2635,6 +2641,47 @@
         <v>60</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B53" t="s">
+        <v>61</v>
+      </c>
+      <c r="C53" t="s">
+        <v>31</v>
+      </c>
+      <c r="D53" t="n">
+        <v>174.887483211358</v>
+      </c>
+      <c r="E53" t="n">
+        <v>57</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="n">
+        <v>443</v>
+      </c>
+      <c r="H53" t="n">
+        <v>96</v>
+      </c>
+      <c r="I53" t="n">
+        <v>347</v>
+      </c>
+      <c r="J53" t="n">
+        <v>12</v>
+      </c>
+      <c r="K53" t="n">
+        <v>3641</v>
+      </c>
+      <c r="L53" t="n">
+        <v>17</v>
+      </c>
+      <c r="M53" t="s">
+        <v>62</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-01]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="66">
   <si>
     <t>date</t>
   </si>
@@ -210,6 +210,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/colombia/primera-b/, /football/el-salvador/primera-division/, /football/estonia/esiliiga/, /football/ethiopia/premier-league/, /football/guatemala/liga-nacional/, /football/latvia/virsliga/, /football/peru/liga-1/, /football/peru/liga-2/, /football/peru/liga-2/, /football/ukraine/premier-league/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bfafc83251cba39ffd730bd8da72e5d134f3e68e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/bulgaria/vtora-liga/, /football/colombia/primera-a/, /football/estonia/esiliiga/, /football/faroe-islands/premier-league/, /football/finland/veikkausliiga/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -2729,6 +2735,47 @@
         <v>64</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B55" t="s">
+        <v>65</v>
+      </c>
+      <c r="C55" t="s">
+        <v>31</v>
+      </c>
+      <c r="D55" t="n">
+        <v>251.282727905114</v>
+      </c>
+      <c r="E55" t="n">
+        <v>69</v>
+      </c>
+      <c r="F55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" t="n">
+        <v>484</v>
+      </c>
+      <c r="H55" t="n">
+        <v>118</v>
+      </c>
+      <c r="I55" t="n">
+        <v>366</v>
+      </c>
+      <c r="J55" t="n">
+        <v>10</v>
+      </c>
+      <c r="K55" t="n">
+        <v>4135</v>
+      </c>
+      <c r="L55" t="n">
+        <v>22</v>
+      </c>
+      <c r="M55" t="s">
+        <v>66</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-02]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="70">
   <si>
     <t>date</t>
   </si>
@@ -222,6 +222,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/luxembourg/bgl-ligue/, /football/poland/ekstraklasa/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a38d2f2cee44ccf7f291acc6b23602a777334dc4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/australia/npl-act/, /football/colombia/primera-a/, /football/faroe-islands/premier-league/, /football/fiji/premier-league/, /football/finland/veikkausliiga/, /football/finland/ykkosliiga/, /football/kazakhstan/premier-league/, /football/south-korea/k-league-1/</t>
   </si>
 </sst>
 </file>
@@ -2823,6 +2829,47 @@
         <v>68</v>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B57" t="s">
+        <v>69</v>
+      </c>
+      <c r="C57" t="s">
+        <v>31</v>
+      </c>
+      <c r="D57" t="n">
+        <v>263.043486662706</v>
+      </c>
+      <c r="E57" t="n">
+        <v>79</v>
+      </c>
+      <c r="F57" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" t="n">
+        <v>491</v>
+      </c>
+      <c r="H57" t="n">
+        <v>143</v>
+      </c>
+      <c r="I57" t="n">
+        <v>348</v>
+      </c>
+      <c r="J57" t="n">
+        <v>31</v>
+      </c>
+      <c r="K57" t="n">
+        <v>4677</v>
+      </c>
+      <c r="L57" t="n">
+        <v>34</v>
+      </c>
+      <c r="M57" t="s">
+        <v>70</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-03]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="74">
   <si>
     <t>date</t>
   </si>
@@ -234,6 +234,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/chile/liga-de-ascenso/, /football/colombia/primera-a/, /football/malawi/super-league/, /football/netherlands/eredivisie/, /football/paraguay/division-intermedia/, /football/romania/liga-2/, /football/sweden/superettan/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b7f5b6bd1cb62fc4fb60be061c1497cda95bafd5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/denmark/1st-division/, /football/ecuador/liga-pro/, /football/ethiopia/premier-league/, /football/faroe-islands/premier-league/, /football/latvia/virsliga/, /football/netherlands/eredivisie/, /football/peru/liga-1/, /football/south-korea/k-league-2/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -2917,6 +2923,47 @@
         <v>72</v>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B59" t="s">
+        <v>73</v>
+      </c>
+      <c r="C59" t="s">
+        <v>31</v>
+      </c>
+      <c r="D59" t="n">
+        <v>255.468648660183</v>
+      </c>
+      <c r="E59" t="n">
+        <v>74</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" t="n">
+        <v>416</v>
+      </c>
+      <c r="H59" t="n">
+        <v>104</v>
+      </c>
+      <c r="I59" t="n">
+        <v>312</v>
+      </c>
+      <c r="J59" t="n">
+        <v>67</v>
+      </c>
+      <c r="K59" t="n">
+        <v>4464</v>
+      </c>
+      <c r="L59" t="n">
+        <v>22</v>
+      </c>
+      <c r="M59" t="s">
+        <v>74</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-04]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="78">
   <si>
     <t>date</t>
   </si>
@@ -246,6 +246,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/2-liga/, /football/bosnia-and-herzegovina/prva-liga-fbih/, /football/croatia/hnl/, /football/greece/super-league/, /football/portugal/liga-portugal-2/, /football/romania/superliga/, /football/south-korea/k-league-2/, /football/sweden/superettan/, /football/ukraine/premier-league/, /football/venezuela/liga-futve-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c5cabee6bfa6e6208caf7163f204ccfbf12bc52e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/croatia/hnl/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/peru/liga-1/, /football/romania/superliga/, /football/slovenia/prva-liga/, /football/sweden/superettan/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -3011,6 +3017,47 @@
         <v>76</v>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B61" t="s">
+        <v>77</v>
+      </c>
+      <c r="C61" t="s">
+        <v>31</v>
+      </c>
+      <c r="D61" t="n">
+        <v>236.764975202084</v>
+      </c>
+      <c r="E61" t="n">
+        <v>58</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" t="n">
+        <v>376</v>
+      </c>
+      <c r="H61" t="n">
+        <v>122</v>
+      </c>
+      <c r="I61" t="n">
+        <v>254</v>
+      </c>
+      <c r="J61" t="n">
+        <v>54</v>
+      </c>
+      <c r="K61" t="n">
+        <v>3780</v>
+      </c>
+      <c r="L61" t="n">
+        <v>18</v>
+      </c>
+      <c r="M61" t="s">
+        <v>78</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-05]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="82">
   <si>
     <t>date</t>
   </si>
@@ -258,6 +258,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/australia/npl-act/, /football/austria/2-liga/, /football/belgium/jupiler-pro-league/, /football/denmark/1st-division/, /football/finland/ykkosliiga/, /football/ireland/division-1/, /football/peru/liga-1/, /football/poland/division-1/, /football/portugal/liga-portugal-2/, /football/portugal/liga-portugal-2/, /football/romania/superliga/, /football/ukraine/premier-league/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">333c642079574ac714ae99749199e1b67a45ec6b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/ecuador/serie-b/, /football/ethiopia/premier-league/, /football/kazakhstan/premier-league/, /football/peru/liga-2/, /football/poland/division-1/, /football/portugal/liga-portugal-2/, /football/romania/superliga/, /football/ukraine/premier-league/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -3105,6 +3111,47 @@
         <v>80</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B63" t="s">
+        <v>81</v>
+      </c>
+      <c r="C63" t="s">
+        <v>31</v>
+      </c>
+      <c r="D63" t="n">
+        <v>272.221403741837</v>
+      </c>
+      <c r="E63" t="n">
+        <v>51</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" t="n">
+        <v>409</v>
+      </c>
+      <c r="H63" t="n">
+        <v>88</v>
+      </c>
+      <c r="I63" t="n">
+        <v>321</v>
+      </c>
+      <c r="J63" t="n">
+        <v>16</v>
+      </c>
+      <c r="K63" t="n">
+        <v>3600</v>
+      </c>
+      <c r="L63" t="n">
+        <v>16</v>
+      </c>
+      <c r="M63" t="s">
+        <v>82</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-06]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="86">
   <si>
     <t>date</t>
   </si>
@@ -270,6 +270,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/egypt/premier-league/, /football/ethiopia/premier-league/, /football/finland/ykkosliiga/, /football/finland/ykkosliiga/, /football/lithuania/i-lyga/, /football/luxembourg/bgl-ligue/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50580dcf4520bfb973e08f23d4f52867142b6b66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/colombia/primera-b/, /football/luxembourg/bgl-ligue/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -3199,6 +3205,47 @@
         <v>84</v>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B65" t="s">
+        <v>85</v>
+      </c>
+      <c r="C65" t="s">
+        <v>31</v>
+      </c>
+      <c r="D65" t="n">
+        <v>209.348263251781</v>
+      </c>
+      <c r="E65" t="n">
+        <v>62</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" t="n">
+        <v>435</v>
+      </c>
+      <c r="H65" t="n">
+        <v>135</v>
+      </c>
+      <c r="I65" t="n">
+        <v>300</v>
+      </c>
+      <c r="J65" t="n">
+        <v>18</v>
+      </c>
+      <c r="K65" t="n">
+        <v>4186</v>
+      </c>
+      <c r="L65" t="n">
+        <v>26</v>
+      </c>
+      <c r="M65" t="s">
+        <v>86</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-07]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="90">
   <si>
     <t>date</t>
   </si>
@@ -282,6 +282,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/ethiopia/premier-league/, /football/faroe-islands/premier-league/, /football/finland/ykkosliiga/, /football/peru/liga-1/, /football/ukraine/premier-league/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f029db27fa38bf89437d058236aeaa8bf8101793</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/belgium/jupiler-pro-league/, /football/faroe-islands/premier-league/, /football/finland/veikkausliiga/, /football/finland/ykkosliiga/, /football/kazakhstan/premier-league/, /football/peru/liga-1/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -3293,6 +3299,47 @@
         <v>88</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B67" t="s">
+        <v>89</v>
+      </c>
+      <c r="C67" t="s">
+        <v>31</v>
+      </c>
+      <c r="D67" t="n">
+        <v>296.931596616904</v>
+      </c>
+      <c r="E67" t="n">
+        <v>58</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" t="n">
+        <v>414</v>
+      </c>
+      <c r="H67" t="n">
+        <v>135</v>
+      </c>
+      <c r="I67" t="n">
+        <v>279</v>
+      </c>
+      <c r="J67" t="n">
+        <v>13</v>
+      </c>
+      <c r="K67" t="n">
+        <v>4012</v>
+      </c>
+      <c r="L67" t="n">
+        <v>23</v>
+      </c>
+      <c r="M67" t="s">
+        <v>90</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-08]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="94">
   <si>
     <t>date</t>
   </si>
@@ -294,6 +294,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/bulgaria/vtora-liga/, /football/peru/liga-1/, /football/peru/liga-2/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">52c4a31cd124150b613d04974982a9abc7024a4c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/estonia/esiliiga/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/peru/liga-1/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -3387,6 +3393,47 @@
         <v>92</v>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B69" t="s">
+        <v>93</v>
+      </c>
+      <c r="C69" t="s">
+        <v>31</v>
+      </c>
+      <c r="D69" t="n">
+        <v>211.704969573021</v>
+      </c>
+      <c r="E69" t="n">
+        <v>67</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" t="n">
+        <v>470</v>
+      </c>
+      <c r="H69" t="n">
+        <v>134</v>
+      </c>
+      <c r="I69" t="n">
+        <v>336</v>
+      </c>
+      <c r="J69" t="n">
+        <v>8</v>
+      </c>
+      <c r="K69" t="n">
+        <v>4349</v>
+      </c>
+      <c r="L69" t="n">
+        <v>27</v>
+      </c>
+      <c r="M69" t="s">
+        <v>94</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-09]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="98">
   <si>
     <t>date</t>
   </si>
@@ -306,6 +306,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/esiliiga/, /football/finland/ykkosliiga/, /football/greece/super-league/, /football/latvia/nakotnes-liga/, /football/lithuania/i-lyga/, /football/romania/superliga/, /football/sweden/superettan/, /football/uruguay/liga-auf-uruguaya/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ef938e70756423463393957b40d144b201fdd8ac</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/ethiopia/premier-league/, /football/finland/veikkausliiga/, /football/greece/super-league/, /football/ireland/division-1/, /football/peru/liga-2/, /football/sweden/superettan/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -3481,6 +3487,47 @@
         <v>96</v>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B71" t="s">
+        <v>97</v>
+      </c>
+      <c r="C71" t="s">
+        <v>31</v>
+      </c>
+      <c r="D71" t="n">
+        <v>252.876885739962</v>
+      </c>
+      <c r="E71" t="n">
+        <v>71</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" t="n">
+        <v>434</v>
+      </c>
+      <c r="H71" t="n">
+        <v>108</v>
+      </c>
+      <c r="I71" t="n">
+        <v>326</v>
+      </c>
+      <c r="J71" t="n">
+        <v>30</v>
+      </c>
+      <c r="K71" t="n">
+        <v>4447</v>
+      </c>
+      <c r="L71" t="n">
+        <v>29</v>
+      </c>
+      <c r="M71" t="s">
+        <v>98</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-10]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="102">
   <si>
     <t>date</t>
   </si>
@@ -318,6 +318,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/belgium/jupiler-pro-league/, /football/cameroon/elite-one/, /football/canada/canadian-premier-league/, /football/colombia/primera-b/, /football/croatia/hnl/, /football/finland/veikkausliiga/, /football/france/ligue-2/, /football/greece/super-league/, /football/peru/liga-1/, /football/ukraine/premier-league/, /football/venezuela/liga-futve-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0de89f56d1cd6088ba6d0a01a49556847f371f8d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/croatia/hnl/, /football/ethiopia/premier-league/, /football/faroe-islands/premier-league/, /football/finland/veikkausliiga/, /football/finland/veikkausliiga/, /football/greece/super-league/, /football/iraq/stars-league/, /football/ireland/premier-division/, /football/malawi/super-league/, /football/south-korea/k-league-2/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -3575,6 +3581,47 @@
         <v>100</v>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B73" t="s">
+        <v>101</v>
+      </c>
+      <c r="C73" t="s">
+        <v>31</v>
+      </c>
+      <c r="D73" t="n">
+        <v>271.948857311408</v>
+      </c>
+      <c r="E73" t="n">
+        <v>65</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" t="n">
+        <v>346</v>
+      </c>
+      <c r="H73" t="n">
+        <v>92</v>
+      </c>
+      <c r="I73" t="n">
+        <v>254</v>
+      </c>
+      <c r="J73" t="n">
+        <v>69</v>
+      </c>
+      <c r="K73" t="n">
+        <v>4423</v>
+      </c>
+      <c r="L73" t="n">
+        <v>22</v>
+      </c>
+      <c r="M73" t="s">
+        <v>102</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-11]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="106">
   <si>
     <t>date</t>
   </si>
@@ -330,6 +330,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/2-liga/, /football/bulgaria/vtora-liga/, /football/finland/veikkausliiga/, /football/greece/super-league/, /football/greece/super-league/, /football/lithuania/i-lyga/, /football/peru/liga-1/, /football/poland/division-1/, /football/portugal/liga-portugal-2/, /football/romania/superliga/, /football/scotland/premiership/, /football/slovenia/prva-liga/, /football/south-korea/k-league-2/, /football/ukraine/premier-league/, /football/venezuela/liga-futve-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">de4257c4cbf52c1535d908bd11d1b7d84895d02a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/finland/veikkausliiga/, /football/finland/ykkosliiga/, /football/lithuania/i-lyga/, /football/slovenia/prva-liga/, /football/south-korea/k-league-2/, /football/sweden/superettan/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -3669,6 +3675,47 @@
         <v>104</v>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B75" t="s">
+        <v>105</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75" t="n">
+        <v>235.447279040019</v>
+      </c>
+      <c r="E75" t="n">
+        <v>51</v>
+      </c>
+      <c r="F75" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" t="n">
+        <v>297</v>
+      </c>
+      <c r="H75" t="n">
+        <v>58</v>
+      </c>
+      <c r="I75" t="n">
+        <v>239</v>
+      </c>
+      <c r="J75" t="n">
+        <v>53</v>
+      </c>
+      <c r="K75" t="n">
+        <v>3834</v>
+      </c>
+      <c r="L75" t="n">
+        <v>12</v>
+      </c>
+      <c r="M75" t="s">
+        <v>106</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-12]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="110">
   <si>
     <t>date</t>
   </si>
@@ -342,6 +342,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/australia/npl-act/, /football/croatia/hnl/, /football/estonia/meistriliiga/, /football/ethiopia/premier-league/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/norway/obos-ligaen/, /football/slovenia/prva-liga/, /football/south-korea/k-league-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cc3976c50592710be763b7e2476d8fdd0bdc8a0f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/canada/canadian-premier-league/, /football/ethiopia/premier-league/, /football/finland/ykkosliiga/, /football/iraq/stars-league/, /football/kazakhstan/premier-league/, /football/south-korea/k-league-2/</t>
   </si>
 </sst>
 </file>
@@ -3763,6 +3769,47 @@
         <v>108</v>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B77" t="s">
+        <v>109</v>
+      </c>
+      <c r="C77" t="s">
+        <v>31</v>
+      </c>
+      <c r="D77" t="n">
+        <v>205.025842555364</v>
+      </c>
+      <c r="E77" t="n">
+        <v>54</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" t="n">
+        <v>395</v>
+      </c>
+      <c r="H77" t="n">
+        <v>85</v>
+      </c>
+      <c r="I77" t="n">
+        <v>310</v>
+      </c>
+      <c r="J77" t="n">
+        <v>9</v>
+      </c>
+      <c r="K77" t="n">
+        <v>4221</v>
+      </c>
+      <c r="L77" t="n">
+        <v>17</v>
+      </c>
+      <c r="M77" t="s">
+        <v>110</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-13]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="114">
   <si>
     <t>date</t>
   </si>
@@ -354,6 +354,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/ethiopia/premier-league/, /football/iraq/stars-league/, /football/lithuania/i-lyga/, /football/mexico/liga-mx/, /football/sweden/superettan/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b27a215410813a47b057f99765297d5cd5197ee8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/cameroon/elite-one/, /football/iraq/stars-league/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/peru/liga-1/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -3857,6 +3863,47 @@
         <v>112</v>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B79" t="s">
+        <v>113</v>
+      </c>
+      <c r="C79" t="s">
+        <v>31</v>
+      </c>
+      <c r="D79" t="n">
+        <v>219.471662461758</v>
+      </c>
+      <c r="E79" t="n">
+        <v>50</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" t="n">
+        <v>359</v>
+      </c>
+      <c r="H79" t="n">
+        <v>79</v>
+      </c>
+      <c r="I79" t="n">
+        <v>280</v>
+      </c>
+      <c r="J79" t="n">
+        <v>6</v>
+      </c>
+      <c r="K79" t="n">
+        <v>3872</v>
+      </c>
+      <c r="L79" t="n">
+        <v>15</v>
+      </c>
+      <c r="M79" t="s">
+        <v>114</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-14]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="118">
   <si>
     <t>date</t>
   </si>
@@ -366,6 +366,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/ecuador/serie-b/, /football/el-salvador/primera-division/, /football/iraq/stars-league/, /football/peru/liga-1/, /football/peru/liga-2/, /football/romania/liga-2/, /football/sweden/superettan/, /football/sweden/superettan/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8ea7fe60d9e8dcc7238dccf611bc4226a532874f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/bulgaria/vtora-liga/, /football/ethiopia/premier-league/, /football/faroe-islands/premier-league/, /football/finland/veikkausliiga/, /football/finland/ykkosliiga/, /football/luxembourg/bgl-ligue/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -3951,6 +3957,47 @@
         <v>116</v>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B81" t="s">
+        <v>117</v>
+      </c>
+      <c r="C81" t="s">
+        <v>31</v>
+      </c>
+      <c r="D81" t="n">
+        <v>238.4404332002</v>
+      </c>
+      <c r="E81" t="n">
+        <v>66</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" t="n">
+        <v>406</v>
+      </c>
+      <c r="H81" t="n">
+        <v>117</v>
+      </c>
+      <c r="I81" t="n">
+        <v>289</v>
+      </c>
+      <c r="J81" t="n">
+        <v>37</v>
+      </c>
+      <c r="K81" t="n">
+        <v>4895</v>
+      </c>
+      <c r="L81" t="n">
+        <v>23</v>
+      </c>
+      <c r="M81" t="s">
+        <v>118</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-15]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="120">
   <si>
     <t>date</t>
   </si>
@@ -372,6 +372,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/bulgaria/vtora-liga/, /football/ethiopia/premier-league/, /football/faroe-islands/premier-league/, /football/finland/veikkausliiga/, /football/finland/ykkosliiga/, /football/luxembourg/bgl-ligue/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e7b9d3cb7d4f08fbe180690c9b81f24c55ecda2a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/armenia/premier-league/, /football/bulgaria/vtora-liga/, /football/kazakhstan/premier-league/, /football/luxembourg/bgl-ligue/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -3998,6 +4004,47 @@
         <v>118</v>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="1" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B82" t="s">
+        <v>119</v>
+      </c>
+      <c r="C82" t="s">
+        <v>31</v>
+      </c>
+      <c r="D82" t="n">
+        <v>171.964472981294</v>
+      </c>
+      <c r="E82" t="n">
+        <v>64</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" t="n">
+        <v>401</v>
+      </c>
+      <c r="H82" t="n">
+        <v>101</v>
+      </c>
+      <c r="I82" t="n">
+        <v>300</v>
+      </c>
+      <c r="J82" t="n">
+        <v>3</v>
+      </c>
+      <c r="K82" t="n">
+        <v>4596</v>
+      </c>
+      <c r="L82" t="n">
+        <v>23</v>
+      </c>
+      <c r="M82" t="s">
+        <v>120</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-16]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="124">
   <si>
     <t>date</t>
   </si>
@@ -384,6 +384,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/meistriliiga/, /football/estonia/esiliiga/, /football/paraguay/division-intermedia/, /football/peru/liga-1/, /football/uruguay/segunda-division/, /football/usa/mls/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e639064ee4f2dc5d32fbba4b45f7a219be05343d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bosnia-and-herzegovina/prva-liga-fbih/, /football/cameroon/elite-one/, /football/estonia/meistriliiga/, /football/estonia/esiliiga/, /football/faroe-islands/premier-league/, /football/norway/obos-ligaen/, /football/peru/liga-1/, /football/portugal/liga-portugal/, /football/ukraine/premier-league/, /football/usa/usl-championship/, /football/venezuela/liga-futve-2/</t>
   </si>
 </sst>
 </file>
@@ -4092,6 +4098,47 @@
         <v>122</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="1" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B84" t="s">
+        <v>123</v>
+      </c>
+      <c r="C84" t="s">
+        <v>31</v>
+      </c>
+      <c r="D84" t="n">
+        <v>253.871300276121</v>
+      </c>
+      <c r="E84" t="n">
+        <v>64</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" t="n">
+        <v>331</v>
+      </c>
+      <c r="H84" t="n">
+        <v>112</v>
+      </c>
+      <c r="I84" t="n">
+        <v>219</v>
+      </c>
+      <c r="J84" t="n">
+        <v>68</v>
+      </c>
+      <c r="K84" t="n">
+        <v>4564</v>
+      </c>
+      <c r="L84" t="n">
+        <v>18</v>
+      </c>
+      <c r="M84" t="s">
+        <v>124</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-17]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="126">
   <si>
     <t>date</t>
   </si>
@@ -390,6 +390,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bosnia-and-herzegovina/prva-liga-fbih/, /football/cameroon/elite-one/, /football/estonia/meistriliiga/, /football/estonia/esiliiga/, /football/faroe-islands/premier-league/, /football/norway/obos-ligaen/, /football/peru/liga-1/, /football/portugal/liga-portugal/, /football/ukraine/premier-league/, /football/usa/usl-championship/, /football/venezuela/liga-futve-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">121dec9bc75e12da09bca04bd202a1b470c415aa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/cameroon/elite-one/, /football/finland/veikkausliiga/, /football/finland/ykkosliiga/, /football/iceland/division-1/, /football/ireland/division-1/, /football/latvia/virsliga/, /football/malawi/super-league/, /football/south-korea/k-league-2/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -4139,6 +4145,47 @@
         <v>124</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="1" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B85" t="s">
+        <v>125</v>
+      </c>
+      <c r="C85" t="s">
+        <v>31</v>
+      </c>
+      <c r="D85" t="n">
+        <v>190.164573367437</v>
+      </c>
+      <c r="E85" t="n">
+        <v>66</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" t="n">
+        <v>332</v>
+      </c>
+      <c r="H85" t="n">
+        <v>99</v>
+      </c>
+      <c r="I85" t="n">
+        <v>233</v>
+      </c>
+      <c r="J85" t="n">
+        <v>59</v>
+      </c>
+      <c r="K85" t="n">
+        <v>4489</v>
+      </c>
+      <c r="L85" t="n">
+        <v>25</v>
+      </c>
+      <c r="M85" t="s">
+        <v>126</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-18]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="130">
   <si>
     <t>date</t>
   </si>
@@ -402,6 +402,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/croatia/hnl/, /football/denmark/superliga/, /football/finland/veikkausliiga/, /football/finland/ykkosliiga/, /football/iceland/besta-deild-karla/, /football/iraq/stars-league/, /football/ireland/division-1/, /football/italy/serie-a/, /football/latvia/virsliga/, /football/moldova/super-liga/, /football/slovenia/prva-liga/, /football/slovenia/prva-liga/, /football/south-korea/k-league-2/, /football/spain/laliga/, /football/ukraine/premier-league/, /football/ukraine/premier-league/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6f307764975b722d25e2e73bb438166be9fd0f9b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/brazil/serie-a-betano/, /football/finland/veikkausliiga/, /football/peru/liga-1/, /football/poland/division-1/, /football/romania/superliga/, /football/romania/superliga/, /football/south-korea/k-league-2/, /football/south-korea/k-league-2/, /football/ukraine/premier-league/, /football/uruguay/liga-auf-uruguaya/</t>
   </si>
 </sst>
 </file>
@@ -4233,6 +4239,47 @@
         <v>128</v>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" s="1" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B87" t="s">
+        <v>129</v>
+      </c>
+      <c r="C87" t="s">
+        <v>31</v>
+      </c>
+      <c r="D87" t="n">
+        <v>245.722572898865</v>
+      </c>
+      <c r="E87" t="n">
+        <v>29</v>
+      </c>
+      <c r="F87" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" t="n">
+        <v>186</v>
+      </c>
+      <c r="H87" t="n">
+        <v>84</v>
+      </c>
+      <c r="I87" t="n">
+        <v>102</v>
+      </c>
+      <c r="J87" t="n">
+        <v>44</v>
+      </c>
+      <c r="K87" t="n">
+        <v>2548</v>
+      </c>
+      <c r="L87" t="n">
+        <v>10</v>
+      </c>
+      <c r="M87" t="s">
+        <v>130</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-19]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="132">
   <si>
     <t>date</t>
   </si>
@@ -408,6 +408,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/brazil/serie-a-betano/, /football/finland/veikkausliiga/, /football/peru/liga-1/, /football/poland/division-1/, /football/romania/superliga/, /football/romania/superliga/, /football/south-korea/k-league-2/, /football/south-korea/k-league-2/, /football/ukraine/premier-league/, /football/uruguay/liga-auf-uruguaya/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9e66dd66becb87095075dbb82e3860b408377e9a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/ethiopia/premier-league/, /football/finland/ykkosliiga/, /football/paraguay/division-intermedia/, /football/paraguay/division-intermedia/, /football/paraguay/division-intermedia/, /football/south-america/copa-sudamericana/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -4280,6 +4286,47 @@
         <v>130</v>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" s="1" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B88" t="s">
+        <v>131</v>
+      </c>
+      <c r="C88" t="s">
+        <v>31</v>
+      </c>
+      <c r="D88" t="n">
+        <v>189.785881356398</v>
+      </c>
+      <c r="E88" t="n">
+        <v>21</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" t="n">
+        <v>139</v>
+      </c>
+      <c r="H88" t="n">
+        <v>68</v>
+      </c>
+      <c r="I88" t="n">
+        <v>71</v>
+      </c>
+      <c r="J88" t="n">
+        <v>19</v>
+      </c>
+      <c r="K88" t="n">
+        <v>1894</v>
+      </c>
+      <c r="L88" t="n">
+        <v>7</v>
+      </c>
+      <c r="M88" t="s">
+        <v>132</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-20]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="136">
   <si>
     <t>date</t>
   </si>
@@ -420,6 +420,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/ethiopia/premier-league/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d2d77677ecc7fa568ea191b473f6a50fc8062d1c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/chile/liga-de-ascenso/, /football/ethiopia/premier-league/, /football/finland/ykkosliiga/, /football/lithuania/i-lyga/, /football/luxembourg/bgl-ligue/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -4374,6 +4380,47 @@
         <v>134</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B90" t="s">
+        <v>135</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90" t="n">
+        <v>205.9566816926</v>
+      </c>
+      <c r="E90" t="n">
+        <v>45</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" t="n">
+        <v>284</v>
+      </c>
+      <c r="H90" t="n">
+        <v>73</v>
+      </c>
+      <c r="I90" t="n">
+        <v>211</v>
+      </c>
+      <c r="J90" t="n">
+        <v>18</v>
+      </c>
+      <c r="K90" t="n">
+        <v>3671</v>
+      </c>
+      <c r="L90" t="n">
+        <v>18</v>
+      </c>
+      <c r="M90" t="s">
+        <v>136</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-21]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="140">
   <si>
     <t>date</t>
   </si>
@@ -432,6 +432,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bosnia-and-herzegovina/prva-liga-fbih/, /football/egypt/premier-league/, /football/ethiopia/premier-league/, /football/faroe-islands/premier-league/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dfb18c71c9586d703d49565ea03ba6a74f5ea2fb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/bosnia-and-herzegovina/prva-liga-fbih/, /football/ecuador/serie-b/, /football/iceland/division-1/, /football/kazakhstan/premier-league/, /football/peru/liga-1/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -4468,6 +4474,47 @@
         <v>138</v>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" s="1" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B92" t="s">
+        <v>139</v>
+      </c>
+      <c r="C92" t="s">
+        <v>31</v>
+      </c>
+      <c r="D92" t="n">
+        <v>163.286817030112</v>
+      </c>
+      <c r="E92" t="n">
+        <v>41</v>
+      </c>
+      <c r="F92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" t="n">
+        <v>252</v>
+      </c>
+      <c r="H92" t="n">
+        <v>65</v>
+      </c>
+      <c r="I92" t="n">
+        <v>187</v>
+      </c>
+      <c r="J92" t="n">
+        <v>17</v>
+      </c>
+      <c r="K92" t="n">
+        <v>3480</v>
+      </c>
+      <c r="L92" t="n">
+        <v>17</v>
+      </c>
+      <c r="M92" t="s">
+        <v>140</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-22]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="144">
   <si>
     <t>date</t>
   </si>
@@ -444,6 +444,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/chile/liga-de-ascenso/, /football/estonia/esiliiga/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/peru/liga-1/, /football/peru/liga-2/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1ce3c272d9989dbc152ef21c804358b472dc3db6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/algeria/ligue-1/, /football/armenia/premier-league/, /football/bulgaria/vtora-liga/, /football/bulgaria/vtora-liga/, /football/chile/liga-de-ascenso/, /football/finland/ykkosliiga/, /football/ireland/division-1/, /football/latvia/virsliga/, /football/uruguay/segunda-division/, /football/venezuela/liga-futve-2/</t>
   </si>
 </sst>
 </file>
@@ -4562,6 +4568,47 @@
         <v>142</v>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" s="1" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B94" t="s">
+        <v>143</v>
+      </c>
+      <c r="C94" t="s">
+        <v>31</v>
+      </c>
+      <c r="D94" t="n">
+        <v>196.300611913204</v>
+      </c>
+      <c r="E94" t="n">
+        <v>50</v>
+      </c>
+      <c r="F94" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94" t="n">
+        <v>329</v>
+      </c>
+      <c r="H94" t="n">
+        <v>137</v>
+      </c>
+      <c r="I94" t="n">
+        <v>192</v>
+      </c>
+      <c r="J94" t="n">
+        <v>19</v>
+      </c>
+      <c r="K94" t="n">
+        <v>3967</v>
+      </c>
+      <c r="L94" t="n">
+        <v>16</v>
+      </c>
+      <c r="M94" t="s">
+        <v>144</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-23]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="146">
   <si>
     <t>date</t>
   </si>
@@ -450,6 +450,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/algeria/ligue-1/, /football/armenia/premier-league/, /football/bulgaria/vtora-liga/, /football/bulgaria/vtora-liga/, /football/chile/liga-de-ascenso/, /football/finland/ykkosliiga/, /football/ireland/division-1/, /football/latvia/virsliga/, /football/uruguay/segunda-division/, /football/venezuela/liga-futve-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">463452443731a52b69ba80a92a50a8be0c6a6792</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/faroe-islands/premier-league/, /football/malawi/super-league/, /football/peru/liga-1/</t>
   </si>
 </sst>
 </file>
@@ -4609,6 +4615,47 @@
         <v>144</v>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" s="1" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B95" t="s">
+        <v>145</v>
+      </c>
+      <c r="C95" t="s">
+        <v>31</v>
+      </c>
+      <c r="D95" t="n">
+        <v>134.832487134139</v>
+      </c>
+      <c r="E95" t="n">
+        <v>55</v>
+      </c>
+      <c r="F95" t="n">
+        <v>0</v>
+      </c>
+      <c r="G95" t="n">
+        <v>314</v>
+      </c>
+      <c r="H95" t="n">
+        <v>79</v>
+      </c>
+      <c r="I95" t="n">
+        <v>235</v>
+      </c>
+      <c r="J95" t="n">
+        <v>16</v>
+      </c>
+      <c r="K95" t="n">
+        <v>4125</v>
+      </c>
+      <c r="L95" t="n">
+        <v>21</v>
+      </c>
+      <c r="M95" t="s">
+        <v>146</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-24]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="150">
   <si>
     <t>date</t>
   </si>
@@ -462,6 +462,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/faroe-islands/premier-league/, /football/finland/veikkausliiga/, /football/ireland/division-1/, /football/latvia/virsliga/, /football/sweden/superettan/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">57ed93f420cf96a5557d1ae0a039dbda73375c0b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/malawi/super-league/, /football/sweden/superettan/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -4703,6 +4709,47 @@
         <v>148</v>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" s="1" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B97" t="s">
+        <v>149</v>
+      </c>
+      <c r="C97" t="s">
+        <v>31</v>
+      </c>
+      <c r="D97" t="n">
+        <v>104.211516845226</v>
+      </c>
+      <c r="E97" t="n">
+        <v>47</v>
+      </c>
+      <c r="F97" t="n">
+        <v>0</v>
+      </c>
+      <c r="G97" t="n">
+        <v>208</v>
+      </c>
+      <c r="H97" t="n">
+        <v>43</v>
+      </c>
+      <c r="I97" t="n">
+        <v>165</v>
+      </c>
+      <c r="J97" t="n">
+        <v>56</v>
+      </c>
+      <c r="K97" t="n">
+        <v>3709</v>
+      </c>
+      <c r="L97" t="n">
+        <v>20</v>
+      </c>
+      <c r="M97" t="s">
+        <v>150</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-25]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="152">
   <si>
     <t>date</t>
   </si>
@@ -468,6 +468,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/malawi/super-league/, /football/sweden/superettan/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6a019a1ed7da40012192924e18b5512ca5506b8c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/armenia/premier-league/, /football/kazakhstan/premier-league/, /football/south-korea/k-league-2/</t>
   </si>
 </sst>
 </file>
@@ -4750,6 +4756,47 @@
         <v>150</v>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" s="1" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B98" t="s">
+        <v>151</v>
+      </c>
+      <c r="C98" t="s">
+        <v>31</v>
+      </c>
+      <c r="D98" t="n">
+        <v>127.328381240368</v>
+      </c>
+      <c r="E98" t="n">
+        <v>30</v>
+      </c>
+      <c r="F98" t="n">
+        <v>0</v>
+      </c>
+      <c r="G98" t="n">
+        <v>175</v>
+      </c>
+      <c r="H98" t="n">
+        <v>93</v>
+      </c>
+      <c r="I98" t="n">
+        <v>82</v>
+      </c>
+      <c r="J98" t="n">
+        <v>79</v>
+      </c>
+      <c r="K98" t="n">
+        <v>2320</v>
+      </c>
+      <c r="L98" t="n">
+        <v>16</v>
+      </c>
+      <c r="M98" t="s">
+        <v>152</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-26]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="156">
   <si>
     <t>date</t>
   </si>
@@ -480,6 +480,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/denmark/1st-division/, /football/ethiopia/premier-league/, /football/georgia/crystalbet-erovnuli-liga/, /football/ireland/division-1/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e56e21a3c83ef216b7c05460024ace410e686f1a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/australia/npl-act/, /football/chile/liga-de-ascenso/, /football/finland/veikkausliiga/, /football/finland/ykkosliiga/, /football/peru/liga-1/, /football/peru/liga-1/</t>
   </si>
 </sst>
 </file>
@@ -4844,6 +4850,47 @@
         <v>154</v>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" s="1" t="n">
+        <v>46168</v>
+      </c>
+      <c r="B100" t="s">
+        <v>155</v>
+      </c>
+      <c r="C100" t="s">
+        <v>31</v>
+      </c>
+      <c r="D100" t="n">
+        <v>128.401276663939</v>
+      </c>
+      <c r="E100" t="n">
+        <v>12</v>
+      </c>
+      <c r="F100" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100" t="n">
+        <v>98</v>
+      </c>
+      <c r="H100" t="n">
+        <v>40</v>
+      </c>
+      <c r="I100" t="n">
+        <v>58</v>
+      </c>
+      <c r="J100" t="n">
+        <v>6</v>
+      </c>
+      <c r="K100" t="n">
+        <v>1276</v>
+      </c>
+      <c r="L100" t="n">
+        <v>5</v>
+      </c>
+      <c r="M100" t="s">
+        <v>156</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-27]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="160">
   <si>
     <t>date</t>
   </si>
@@ -492,6 +492,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/canada/canadian-premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">93c6746cfdf89d0fb60bd95785a91d663f4ed806</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/ethiopia/premier-league/, /football/kazakhstan/premier-league/, /football/lithuania/i-lyga/, /football/peru/liga-1/, /football/peru/liga-2/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -4938,6 +4944,47 @@
         <v>158</v>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" s="1" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B102" t="s">
+        <v>159</v>
+      </c>
+      <c r="C102" t="s">
+        <v>31</v>
+      </c>
+      <c r="D102" t="n">
+        <v>164.912532715003</v>
+      </c>
+      <c r="E102" t="n">
+        <v>28</v>
+      </c>
+      <c r="F102" t="n">
+        <v>0</v>
+      </c>
+      <c r="G102" t="n">
+        <v>170</v>
+      </c>
+      <c r="H102" t="n">
+        <v>83</v>
+      </c>
+      <c r="I102" t="n">
+        <v>87</v>
+      </c>
+      <c r="J102" t="n">
+        <v>14</v>
+      </c>
+      <c r="K102" t="n">
+        <v>2498</v>
+      </c>
+      <c r="L102" t="n">
+        <v>15</v>
+      </c>
+      <c r="M102" t="s">
+        <v>160</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-28]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="164">
   <si>
     <t>date</t>
   </si>
@@ -504,6 +504,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/australia/npl-act/, /football/belarus/vysshaya-liga/, /football/estonia/esiliiga/, /football/ethiopia/premier-league/, /football/faroe-islands/premier-league/, /football/iceland/division-1/, /football/iraq/stars-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cc4ebf563d9d328b11f80764d6cc7a0abf60abd0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/ecuador/serie-b/, /football/ecuador/serie-b/, /football/ethiopia/premier-league/, /football/georgia/crystalbet-erovnuli-liga/, /football/uruguay/segunda-division/, /football/usa/usl-championship/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -5032,6 +5038,47 @@
         <v>162</v>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" s="1" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B104" t="s">
+        <v>163</v>
+      </c>
+      <c r="C104" t="s">
+        <v>31</v>
+      </c>
+      <c r="D104" t="n">
+        <v>163.708220744133</v>
+      </c>
+      <c r="E104" t="n">
+        <v>29</v>
+      </c>
+      <c r="F104" t="n">
+        <v>0</v>
+      </c>
+      <c r="G104" t="n">
+        <v>164</v>
+      </c>
+      <c r="H104" t="n">
+        <v>70</v>
+      </c>
+      <c r="I104" t="n">
+        <v>94</v>
+      </c>
+      <c r="J104" t="n">
+        <v>15</v>
+      </c>
+      <c r="K104" t="n">
+        <v>2696</v>
+      </c>
+      <c r="L104" t="n">
+        <v>12</v>
+      </c>
+      <c r="M104" t="s">
+        <v>164</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-29]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="168">
   <si>
     <t>date</t>
   </si>
@@ -516,6 +516,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/ecuador/serie-b/, /football/ethiopia/premier-league/, /football/faroe-islands/premier-league/, /football/finland/ykkosliiga/, /football/lithuania/i-lyga/, /football/peru/liga-1/, /football/uruguay/segunda-division/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">54563cbd0018006ed82d5cd3c22412328c285af2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/lithuania/i-lyga/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -5126,6 +5132,47 @@
         <v>166</v>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" s="1" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B106" t="s">
+        <v>167</v>
+      </c>
+      <c r="C106" t="s">
+        <v>31</v>
+      </c>
+      <c r="D106" t="n">
+        <v>86.5811426003774</v>
+      </c>
+      <c r="E106" t="n">
+        <v>31</v>
+      </c>
+      <c r="F106" t="n">
+        <v>0</v>
+      </c>
+      <c r="G106" t="n">
+        <v>172</v>
+      </c>
+      <c r="H106" t="n">
+        <v>75</v>
+      </c>
+      <c r="I106" t="n">
+        <v>97</v>
+      </c>
+      <c r="J106" t="n">
+        <v>6</v>
+      </c>
+      <c r="K106" t="n">
+        <v>2549</v>
+      </c>
+      <c r="L106" t="n">
+        <v>16</v>
+      </c>
+      <c r="M106" t="s">
+        <v>168</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-30]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="172">
   <si>
     <t>date</t>
   </si>
@@ -528,6 +528,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/chile/liga-de-ascenso/, /football/ireland/division-1/, /football/south-america/copa-libertadores/, /football/south-america/copa-sudamericana/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">af318a3851e6bc2a51feae36bc546af4cb0a7c30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/australia/npl-act/, /football/malawi/super-league/, /football/paraguay/division-intermedia/</t>
   </si>
 </sst>
 </file>
@@ -5220,6 +5226,47 @@
         <v>170</v>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" s="1" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B108" t="s">
+        <v>171</v>
+      </c>
+      <c r="C108" t="s">
+        <v>31</v>
+      </c>
+      <c r="D108" t="n">
+        <v>108.391859674454</v>
+      </c>
+      <c r="E108" t="n">
+        <v>37</v>
+      </c>
+      <c r="F108" t="n">
+        <v>0</v>
+      </c>
+      <c r="G108" t="n">
+        <v>167</v>
+      </c>
+      <c r="H108" t="n">
+        <v>66</v>
+      </c>
+      <c r="I108" t="n">
+        <v>101</v>
+      </c>
+      <c r="J108" t="n">
+        <v>14</v>
+      </c>
+      <c r="K108" t="n">
+        <v>2685</v>
+      </c>
+      <c r="L108" t="n">
+        <v>19</v>
+      </c>
+      <c r="M108" t="s">
+        <v>172</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-05-31]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="176">
   <si>
     <t>date</t>
   </si>
@@ -540,6 +540,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/iraq/stars-league/, /football/paraguay/division-intermedia/, /football/venezuela/liga-futve-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">266172fd256c0250d280c7cff11019422b45a1e5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/malawi/super-league/, /football/sierra-leone/premier-league/, /football/south-korea/k-league-2/</t>
   </si>
 </sst>
 </file>
@@ -5314,6 +5320,47 @@
         <v>174</v>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" s="1" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B110" t="s">
+        <v>175</v>
+      </c>
+      <c r="C110" t="s">
+        <v>31</v>
+      </c>
+      <c r="D110" t="n">
+        <v>88.8963738679886</v>
+      </c>
+      <c r="E110" t="n">
+        <v>31</v>
+      </c>
+      <c r="F110" t="n">
+        <v>0</v>
+      </c>
+      <c r="G110" t="n">
+        <v>92</v>
+      </c>
+      <c r="H110" t="n">
+        <v>30</v>
+      </c>
+      <c r="I110" t="n">
+        <v>62</v>
+      </c>
+      <c r="J110" t="n">
+        <v>16</v>
+      </c>
+      <c r="K110" t="n">
+        <v>2556</v>
+      </c>
+      <c r="L110" t="n">
+        <v>13</v>
+      </c>
+      <c r="M110" t="s">
+        <v>176</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-01]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="180">
   <si>
     <t>date</t>
   </si>
@@ -552,6 +552,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/norway/obos-ligaen/, /football/peru/liga-2/, /football/sierra-leone/premier-league/, /football/south-korea/k-league-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9eb71997148edb2b30bbd2e5b5e5a0172d978892</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/iraq/stars-league/, /football/south-korea/k-league-2/</t>
   </si>
 </sst>
 </file>
@@ -5408,6 +5414,47 @@
         <v>178</v>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B112" t="s">
+        <v>179</v>
+      </c>
+      <c r="C112" t="s">
+        <v>31</v>
+      </c>
+      <c r="D112" t="n">
+        <v>97.9183407266935</v>
+      </c>
+      <c r="E112" t="n">
+        <v>13</v>
+      </c>
+      <c r="F112" t="n">
+        <v>0</v>
+      </c>
+      <c r="G112" t="n">
+        <v>40</v>
+      </c>
+      <c r="H112" t="n">
+        <v>33</v>
+      </c>
+      <c r="I112" t="n">
+        <v>7</v>
+      </c>
+      <c r="J112" t="n">
+        <v>32</v>
+      </c>
+      <c r="K112" t="n">
+        <v>857</v>
+      </c>
+      <c r="L112" t="n">
+        <v>9</v>
+      </c>
+      <c r="M112" t="s">
+        <v>180</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-02]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="184">
   <si>
     <t>date</t>
   </si>
@@ -564,6 +564,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/south-korea/k-league-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b18d18a803454b2997ce345d5de310269680095c</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
   </si>
 </sst>
 </file>
@@ -5502,6 +5508,47 @@
         <v>182</v>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" s="1" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B114" t="s">
+        <v>183</v>
+      </c>
+      <c r="C114" t="s">
+        <v>31</v>
+      </c>
+      <c r="D114" t="n">
+        <v>56.5328705708186</v>
+      </c>
+      <c r="E114" t="n">
+        <v>13</v>
+      </c>
+      <c r="F114" t="n">
+        <v>0</v>
+      </c>
+      <c r="G114" t="n">
+        <v>58</v>
+      </c>
+      <c r="H114" t="n">
+        <v>49</v>
+      </c>
+      <c r="I114" t="n">
+        <v>9</v>
+      </c>
+      <c r="J114" t="n">
+        <v>4</v>
+      </c>
+      <c r="K114" t="n">
+        <v>1315</v>
+      </c>
+      <c r="L114" t="n">
+        <v>8</v>
+      </c>
+      <c r="M114" t="s">
+        <v>184</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-03]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="188">
   <si>
     <t>date</t>
   </si>
@@ -576,6 +576,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/cameroon/elite-one/, /football/ecuador/serie-b/, /football/ireland/premier-division/, /football/sweden/superettan/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">63d8813c932377bdc10768b942b35119e00841f1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/chile/liga-de-primera/, /football/chile/liga-de-ascenso/, /football/ireland/premier-division/, /football/sweden/superettan/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -5596,6 +5602,47 @@
         <v>186</v>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" s="1" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B116" t="s">
+        <v>187</v>
+      </c>
+      <c r="C116" t="s">
+        <v>31</v>
+      </c>
+      <c r="D116" t="n">
+        <v>112.266016145547</v>
+      </c>
+      <c r="E116" t="n">
+        <v>9</v>
+      </c>
+      <c r="F116" t="n">
+        <v>0</v>
+      </c>
+      <c r="G116" t="n">
+        <v>35</v>
+      </c>
+      <c r="H116" t="n">
+        <v>21</v>
+      </c>
+      <c r="I116" t="n">
+        <v>14</v>
+      </c>
+      <c r="J116" t="n">
+        <v>0</v>
+      </c>
+      <c r="K116" t="n">
+        <v>966</v>
+      </c>
+      <c r="L116" t="n">
+        <v>4</v>
+      </c>
+      <c r="M116" t="s">
+        <v>188</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-04]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="192">
   <si>
     <t>date</t>
   </si>
@@ -588,6 +588,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/meistriliiga/, /football/finland/veikkausliiga/, /football/ireland/premier-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f39094609f9e7d787a7389332e14951a360c06e3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/cameroon/elite-one/, /football/chile/liga-de-primera/, /football/estonia/meistriliiga/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -5690,6 +5696,47 @@
         <v>190</v>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" s="1" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B118" t="s">
+        <v>191</v>
+      </c>
+      <c r="C118" t="s">
+        <v>31</v>
+      </c>
+      <c r="D118" t="n">
+        <v>105.354630068938</v>
+      </c>
+      <c r="E118" t="n">
+        <v>10</v>
+      </c>
+      <c r="F118" t="n">
+        <v>0</v>
+      </c>
+      <c r="G118" t="n">
+        <v>42</v>
+      </c>
+      <c r="H118" t="n">
+        <v>27</v>
+      </c>
+      <c r="I118" t="n">
+        <v>15</v>
+      </c>
+      <c r="J118" t="n">
+        <v>1</v>
+      </c>
+      <c r="K118" t="n">
+        <v>998</v>
+      </c>
+      <c r="L118" t="n">
+        <v>7</v>
+      </c>
+      <c r="M118" t="s">
+        <v>192</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-05]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="196">
   <si>
     <t>date</t>
   </si>
@@ -600,6 +600,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/meistriliiga/, /football/finland/veikkausliiga/, /football/lithuania/i-lyga/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fad3f0e59c506f6fad11c83bc3be14ff56bcad07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/algeria/ligue-1/, /football/ecuador/serie-b/, /football/estonia/meistriliiga/, /football/finland/veikkausliiga/, /football/finland/ykkosliiga/, /football/ireland/premier-division/</t>
   </si>
 </sst>
 </file>
@@ -5784,6 +5790,47 @@
         <v>194</v>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" s="1" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B120" t="s">
+        <v>195</v>
+      </c>
+      <c r="C120" t="s">
+        <v>31</v>
+      </c>
+      <c r="D120" t="n">
+        <v>101.149061536789</v>
+      </c>
+      <c r="E120" t="n">
+        <v>10</v>
+      </c>
+      <c r="F120" t="n">
+        <v>0</v>
+      </c>
+      <c r="G120" t="n">
+        <v>47</v>
+      </c>
+      <c r="H120" t="n">
+        <v>30</v>
+      </c>
+      <c r="I120" t="n">
+        <v>17</v>
+      </c>
+      <c r="J120" t="n">
+        <v>0</v>
+      </c>
+      <c r="K120" t="n">
+        <v>1023</v>
+      </c>
+      <c r="L120" t="n">
+        <v>7</v>
+      </c>
+      <c r="M120" t="s">
+        <v>196</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-06]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="200">
   <si>
     <t>date</t>
   </si>
@@ -612,6 +612,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bosnia-and-herzegovina/prva-liga-fbih/, /football/chile/liga-de-primera/, /football/estonia/meistriliiga/, /football/finland/veikkausliiga/, /football/ireland/premier-division/, /football/lithuania/i-lyga/, /football/paraguay/division-intermedia/, /football/sweden/superettan/, /football/uruguay/segunda-division/, /football/usa/usl-championship/, /football/venezuela/liga-futve-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0e901faca2f1d754818514910964fdeb3c09e94c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/australia/npl-act/, /football/bosnia-and-herzegovina/prva-liga-fbih/, /football/ecuador/liga-pro/, /football/finland/veikkausliiga/, /football/finland/ykkosliiga/, /football/ireland/premier-division/, /football/sweden/superettan/, /football/uruguay/liga-auf-uruguaya/, /football/uruguay/segunda-division/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -5878,6 +5884,47 @@
         <v>198</v>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" s="1" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B122" t="s">
+        <v>199</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122" t="n">
+        <v>146.448560770353</v>
+      </c>
+      <c r="E122" t="n">
+        <v>10</v>
+      </c>
+      <c r="F122" t="n">
+        <v>0</v>
+      </c>
+      <c r="G122" t="n">
+        <v>29</v>
+      </c>
+      <c r="H122" t="n">
+        <v>20</v>
+      </c>
+      <c r="I122" t="n">
+        <v>9</v>
+      </c>
+      <c r="J122" t="n">
+        <v>3</v>
+      </c>
+      <c r="K122" t="n">
+        <v>752</v>
+      </c>
+      <c r="L122" t="n">
+        <v>7</v>
+      </c>
+      <c r="M122" t="s">
+        <v>200</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-07]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="204">
   <si>
     <t>date</t>
   </si>
@@ -624,6 +624,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/australia/npl-act/, /football/ireland/division-1/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">af27af3399dc1ffc2ccdcaa89d9e696b30059b21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/australia/npl-act/, /football/belarus/vysshaya-liga/, /football/ireland/division-1/, /football/kazakhstan/premier-league/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -5972,6 +5978,47 @@
         <v>202</v>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" s="1" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B124" t="s">
+        <v>203</v>
+      </c>
+      <c r="C124" t="s">
+        <v>31</v>
+      </c>
+      <c r="D124" t="n">
+        <v>122.043572167555</v>
+      </c>
+      <c r="E124" t="n">
+        <v>15</v>
+      </c>
+      <c r="F124" t="n">
+        <v>0</v>
+      </c>
+      <c r="G124" t="n">
+        <v>63</v>
+      </c>
+      <c r="H124" t="n">
+        <v>38</v>
+      </c>
+      <c r="I124" t="n">
+        <v>25</v>
+      </c>
+      <c r="J124" t="n">
+        <v>8</v>
+      </c>
+      <c r="K124" t="n">
+        <v>1382</v>
+      </c>
+      <c r="L124" t="n">
+        <v>8</v>
+      </c>
+      <c r="M124" t="s">
+        <v>204</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-08]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="208">
   <si>
     <t>date</t>
   </si>
@@ -636,6 +636,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/australia/npl-act/, /football/bosnia-and-herzegovina/prva-liga-fbih/, /football/estonia/meistriliiga/, /football/finland/ykkosliiga/, /football/lithuania/i-lyga/, /football/norway/obos-ligaen/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abde3ab8060cbc269a48f934ea5ecf59156b6356</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/finland/ykkosliiga/, /football/kazakhstan/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -6066,6 +6072,47 @@
         <v>206</v>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" s="1" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B126" t="s">
+        <v>207</v>
+      </c>
+      <c r="C126" t="s">
+        <v>31</v>
+      </c>
+      <c r="D126" t="n">
+        <v>113.481233795484</v>
+      </c>
+      <c r="E126" t="n">
+        <v>13</v>
+      </c>
+      <c r="F126" t="n">
+        <v>0</v>
+      </c>
+      <c r="G126" t="n">
+        <v>66</v>
+      </c>
+      <c r="H126" t="n">
+        <v>54</v>
+      </c>
+      <c r="I126" t="n">
+        <v>12</v>
+      </c>
+      <c r="J126" t="n">
+        <v>13</v>
+      </c>
+      <c r="K126" t="n">
+        <v>1260</v>
+      </c>
+      <c r="L126" t="n">
+        <v>7</v>
+      </c>
+      <c r="M126" t="s">
+        <v>208</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-09]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="212">
   <si>
     <t>date</t>
   </si>
@@ -648,6 +648,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/canada/canadian-premier-league/, /football/estonia/meistriliiga/, /football/finland/veikkausliiga/, /football/kazakhstan/premier-league/, /football/lithuania/i-lyga/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">541a2bf2cad1204b95f5e3c617898337c57039cb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/canada/canadian-premier-league/, /football/kazakhstan/premier-league/, /football/lithuania/i-lyga/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -6160,6 +6166,47 @@
         <v>210</v>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" s="1" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B128" t="s">
+        <v>211</v>
+      </c>
+      <c r="C128" t="s">
+        <v>31</v>
+      </c>
+      <c r="D128" t="n">
+        <v>96.9297601620356</v>
+      </c>
+      <c r="E128" t="n">
+        <v>13</v>
+      </c>
+      <c r="F128" t="n">
+        <v>0</v>
+      </c>
+      <c r="G128" t="n">
+        <v>80</v>
+      </c>
+      <c r="H128" t="n">
+        <v>34</v>
+      </c>
+      <c r="I128" t="n">
+        <v>46</v>
+      </c>
+      <c r="J128" t="n">
+        <v>1</v>
+      </c>
+      <c r="K128" t="n">
+        <v>1174</v>
+      </c>
+      <c r="L128" t="n">
+        <v>7</v>
+      </c>
+      <c r="M128" t="s">
+        <v>212</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-10]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="216">
   <si>
     <t>date</t>
   </si>
@@ -660,6 +660,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/sweden/superettan/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9c1fe2c8ca823c888259933367e41dabaf048d46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/iceland/division-1/, /football/sweden/superettan/, /football/sweden/superettan/, /football/uruguay/segunda-division/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -6254,6 +6260,47 @@
         <v>214</v>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" s="1" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B130" t="s">
+        <v>215</v>
+      </c>
+      <c r="C130" t="s">
+        <v>31</v>
+      </c>
+      <c r="D130" t="n">
+        <v>116.569607631365</v>
+      </c>
+      <c r="E130" t="n">
+        <v>17</v>
+      </c>
+      <c r="F130" t="n">
+        <v>0</v>
+      </c>
+      <c r="G130" t="n">
+        <v>96</v>
+      </c>
+      <c r="H130" t="n">
+        <v>35</v>
+      </c>
+      <c r="I130" t="n">
+        <v>61</v>
+      </c>
+      <c r="J130" t="n">
+        <v>6</v>
+      </c>
+      <c r="K130" t="n">
+        <v>1450</v>
+      </c>
+      <c r="L130" t="n">
+        <v>6</v>
+      </c>
+      <c r="M130" t="s">
+        <v>216</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-11]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="220">
   <si>
     <t>date</t>
   </si>
@@ -672,6 +672,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/cameroon/elite-one/, /football/kazakhstan/premier-league/, /football/lithuania/i-lyga/, /football/uruguay/segunda-division/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e4e6315eb213ed22ef4a7fefef7ec5d2d6de2ae9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/iceland/division-1/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -6348,6 +6354,47 @@
         <v>218</v>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" s="1" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B132" t="s">
+        <v>219</v>
+      </c>
+      <c r="C132" t="s">
+        <v>31</v>
+      </c>
+      <c r="D132" t="n">
+        <v>112.958818042278</v>
+      </c>
+      <c r="E132" t="n">
+        <v>17</v>
+      </c>
+      <c r="F132" t="n">
+        <v>0</v>
+      </c>
+      <c r="G132" t="n">
+        <v>98</v>
+      </c>
+      <c r="H132" t="n">
+        <v>37</v>
+      </c>
+      <c r="I132" t="n">
+        <v>61</v>
+      </c>
+      <c r="J132" t="n">
+        <v>0</v>
+      </c>
+      <c r="K132" t="n">
+        <v>1405</v>
+      </c>
+      <c r="L132" t="n">
+        <v>9</v>
+      </c>
+      <c r="M132" t="s">
+        <v>220</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-12]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="224">
   <si>
     <t>date</t>
   </si>
@@ -684,6 +684,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/ethiopia/premier-league/, /football/finland/veikkausliiga/, /football/finland/ykkosliiga/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5416acb7858c3b0d6d1df942094b9ea16a80373a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/cameroon/elite-one/, /football/ethiopia/premier-league/, /football/faroe-islands/premier-league/, /football/finland/ykkosliiga/, /football/kazakhstan/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -6442,6 +6448,47 @@
         <v>222</v>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" s="1" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B134" t="s">
+        <v>223</v>
+      </c>
+      <c r="C134" t="s">
+        <v>31</v>
+      </c>
+      <c r="D134" t="n">
+        <v>115.375900308291</v>
+      </c>
+      <c r="E134" t="n">
+        <v>21</v>
+      </c>
+      <c r="F134" t="n">
+        <v>0</v>
+      </c>
+      <c r="G134" t="n">
+        <v>129</v>
+      </c>
+      <c r="H134" t="n">
+        <v>66</v>
+      </c>
+      <c r="I134" t="n">
+        <v>63</v>
+      </c>
+      <c r="J134" t="n">
+        <v>0</v>
+      </c>
+      <c r="K134" t="n">
+        <v>1643</v>
+      </c>
+      <c r="L134" t="n">
+        <v>13</v>
+      </c>
+      <c r="M134" t="s">
+        <v>224</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-13]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="228">
   <si>
     <t>date</t>
   </si>
@@ -696,6 +696,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/latvia/virsliga/, /football/sierra-leone/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">08f23766e4c6867c9f973ade86ba5c2dfb8eb5d9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/cameroon/elite-one/, /football/cameroon/elite-one/, /football/ireland/premier-division/, /football/ireland/division-1/, /football/latvia/nakotnes-liga/, /football/sierra-leone/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -6536,6 +6542,47 @@
         <v>226</v>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B136" t="s">
+        <v>227</v>
+      </c>
+      <c r="C136" t="s">
+        <v>31</v>
+      </c>
+      <c r="D136" t="n">
+        <v>115.307489661376</v>
+      </c>
+      <c r="E136" t="n">
+        <v>25</v>
+      </c>
+      <c r="F136" t="n">
+        <v>0</v>
+      </c>
+      <c r="G136" t="n">
+        <v>124</v>
+      </c>
+      <c r="H136" t="n">
+        <v>63</v>
+      </c>
+      <c r="I136" t="n">
+        <v>61</v>
+      </c>
+      <c r="J136" t="n">
+        <v>6</v>
+      </c>
+      <c r="K136" t="n">
+        <v>1714</v>
+      </c>
+      <c r="L136" t="n">
+        <v>15</v>
+      </c>
+      <c r="M136" t="s">
+        <v>228</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-14]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="232">
   <si>
     <t>date</t>
   </si>
@@ -708,6 +708,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/cameroon/elite-one/, /football/iceland/division-1/, /football/ireland/premier-division/, /football/ireland/division-1/, /football/latvia/virsliga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">499d698fb69e9c67fe63da3a79e42b879cf55359</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/ethiopia/premier-league/, /football/faroe-islands/premier-league/, /football/iceland/division-1/, /football/ireland/premier-division/, /football/ireland/premier-division/, /football/ireland/division-1/, /football/latvia/virsliga/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -6630,6 +6636,47 @@
         <v>230</v>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" s="1" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B138" t="s">
+        <v>231</v>
+      </c>
+      <c r="C138" t="s">
+        <v>31</v>
+      </c>
+      <c r="D138" t="n">
+        <v>126.831220503648</v>
+      </c>
+      <c r="E138" t="n">
+        <v>19</v>
+      </c>
+      <c r="F138" t="n">
+        <v>0</v>
+      </c>
+      <c r="G138" t="n">
+        <v>74</v>
+      </c>
+      <c r="H138" t="n">
+        <v>32</v>
+      </c>
+      <c r="I138" t="n">
+        <v>42</v>
+      </c>
+      <c r="J138" t="n">
+        <v>16</v>
+      </c>
+      <c r="K138" t="n">
+        <v>1385</v>
+      </c>
+      <c r="L138" t="n">
+        <v>11</v>
+      </c>
+      <c r="M138" t="s">
+        <v>232</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-15]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="234">
   <si>
     <t>date</t>
   </si>
@@ -714,6 +714,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/ethiopia/premier-league/, /football/faroe-islands/premier-league/, /football/iceland/division-1/, /football/ireland/premier-division/, /football/ireland/premier-division/, /football/ireland/division-1/, /football/latvia/virsliga/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cc3f26e986e4737ec354a8e62c27b326a2789272</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/italy/serie-a/, /football/sweden/superettan/</t>
   </si>
 </sst>
 </file>
@@ -6677,6 +6683,47 @@
         <v>232</v>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B139" t="s">
+        <v>233</v>
+      </c>
+      <c r="C139" t="s">
+        <v>31</v>
+      </c>
+      <c r="D139" t="n">
+        <v>93.353821070989</v>
+      </c>
+      <c r="E139" t="n">
+        <v>12</v>
+      </c>
+      <c r="F139" t="n">
+        <v>0</v>
+      </c>
+      <c r="G139" t="n">
+        <v>57</v>
+      </c>
+      <c r="H139" t="n">
+        <v>37</v>
+      </c>
+      <c r="I139" t="n">
+        <v>20</v>
+      </c>
+      <c r="J139" t="n">
+        <v>30</v>
+      </c>
+      <c r="K139" t="n">
+        <v>1165</v>
+      </c>
+      <c r="L139" t="n">
+        <v>6</v>
+      </c>
+      <c r="M139" t="s">
+        <v>234</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-16]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="238">
   <si>
     <t>date</t>
   </si>
@@ -726,6 +726,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/esiliiga/, /football/italy/serie-a/, /football/italy/serie-a/, /football/kazakhstan/premier-league/, /football/sweden/superettan/, /football/sweden/superettan/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1bcca12343b9588e71244f5e46708432e523ed4b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/estonia/esiliiga/, /football/finland/veikkausliiga/, /football/ireland/division-1/, /football/italy/serie-a/, /football/latvia/virsliga/</t>
   </si>
 </sst>
 </file>
@@ -6771,6 +6777,47 @@
         <v>236</v>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" s="1" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B141" t="s">
+        <v>237</v>
+      </c>
+      <c r="C141" t="s">
+        <v>31</v>
+      </c>
+      <c r="D141" t="n">
+        <v>95.7258117874463</v>
+      </c>
+      <c r="E141" t="n">
+        <v>14</v>
+      </c>
+      <c r="F141" t="n">
+        <v>0</v>
+      </c>
+      <c r="G141" t="n">
+        <v>83</v>
+      </c>
+      <c r="H141" t="n">
+        <v>57</v>
+      </c>
+      <c r="I141" t="n">
+        <v>26</v>
+      </c>
+      <c r="J141" t="n">
+        <v>1</v>
+      </c>
+      <c r="K141" t="n">
+        <v>1339</v>
+      </c>
+      <c r="L141" t="n">
+        <v>10</v>
+      </c>
+      <c r="M141" t="s">
+        <v>238</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-17]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="242">
   <si>
     <t>date</t>
   </si>
@@ -738,6 +738,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/estonia/esiliiga/, /football/italy/serie-a/, /football/kazakhstan/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a242e4a5b8c44b4c2ebfb1724d3653a99ea757b8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -6865,6 +6871,47 @@
         <v>240</v>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" s="1" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B143" t="s">
+        <v>241</v>
+      </c>
+      <c r="C143" t="s">
+        <v>31</v>
+      </c>
+      <c r="D143" t="n">
+        <v>58.3689425230026</v>
+      </c>
+      <c r="E143" t="n">
+        <v>18</v>
+      </c>
+      <c r="F143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G143" t="n">
+        <v>101</v>
+      </c>
+      <c r="H143" t="n">
+        <v>64</v>
+      </c>
+      <c r="I143" t="n">
+        <v>37</v>
+      </c>
+      <c r="J143" t="n">
+        <v>4</v>
+      </c>
+      <c r="K143" t="n">
+        <v>1591</v>
+      </c>
+      <c r="L143" t="n">
+        <v>12</v>
+      </c>
+      <c r="M143" t="s">
+        <v>242</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-18]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="246">
   <si>
     <t>date</t>
   </si>
@@ -750,6 +750,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/estonia/meistriliiga/, /football/estonia/esiliiga/, /football/finland/veikkausliiga/, /football/iceland/division-1/, /football/italy/serie-a/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2673d14c0ed43c743213efb74ffabf2315bfe7d3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/italy/serie-a/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -6959,6 +6965,47 @@
         <v>244</v>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" s="1" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B145" t="s">
+        <v>245</v>
+      </c>
+      <c r="C145" t="s">
+        <v>31</v>
+      </c>
+      <c r="D145" t="n">
+        <v>69.8000477830569</v>
+      </c>
+      <c r="E145" t="n">
+        <v>17</v>
+      </c>
+      <c r="F145" t="n">
+        <v>0</v>
+      </c>
+      <c r="G145" t="n">
+        <v>88</v>
+      </c>
+      <c r="H145" t="n">
+        <v>60</v>
+      </c>
+      <c r="I145" t="n">
+        <v>28</v>
+      </c>
+      <c r="J145" t="n">
+        <v>5</v>
+      </c>
+      <c r="K145" t="n">
+        <v>1496</v>
+      </c>
+      <c r="L145" t="n">
+        <v>11</v>
+      </c>
+      <c r="M145" t="s">
+        <v>246</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-19]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="249">
   <si>
     <t>date</t>
   </si>
@@ -759,6 +759,12 @@
   </si>
   <si>
     <t xml:space="preserve">c3b0bc3f11e59f5ee6dca48d3507cabb4213dccc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ebf1545c4dbf8e18489a8f767f2b2e5166d64ca5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/pershaya-liga/, /football/iceland/division-1/, /football/lithuania/i-lyga/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -7050,6 +7056,47 @@
         <v>184</v>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" s="1" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B147" t="s">
+        <v>248</v>
+      </c>
+      <c r="C147" t="s">
+        <v>31</v>
+      </c>
+      <c r="D147" t="n">
+        <v>111.620138494174</v>
+      </c>
+      <c r="E147" t="n">
+        <v>21</v>
+      </c>
+      <c r="F147" t="n">
+        <v>0</v>
+      </c>
+      <c r="G147" t="n">
+        <v>120</v>
+      </c>
+      <c r="H147" t="n">
+        <v>67</v>
+      </c>
+      <c r="I147" t="n">
+        <v>53</v>
+      </c>
+      <c r="J147" t="n">
+        <v>1</v>
+      </c>
+      <c r="K147" t="n">
+        <v>1731</v>
+      </c>
+      <c r="L147" t="n">
+        <v>13</v>
+      </c>
+      <c r="M147" t="s">
+        <v>249</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-20]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="253">
   <si>
     <t>date</t>
   </si>
@@ -771,6 +771,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/esiliiga/, /football/iceland/division-1/, /football/mexico/liga-mx/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2b07b390b32c120d76a27b771940fe5519ab938a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/pershaya-liga/, /football/ireland/premier-division/, /football/ireland/premier-division/, /football/malawi/super-league/</t>
   </si>
 </sst>
 </file>
@@ -7144,6 +7150,47 @@
         <v>251</v>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" s="1" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B149" t="s">
+        <v>252</v>
+      </c>
+      <c r="C149" t="s">
+        <v>31</v>
+      </c>
+      <c r="D149" t="n">
+        <v>112.165060067177</v>
+      </c>
+      <c r="E149" t="n">
+        <v>21</v>
+      </c>
+      <c r="F149" t="n">
+        <v>0</v>
+      </c>
+      <c r="G149" t="n">
+        <v>118</v>
+      </c>
+      <c r="H149" t="n">
+        <v>56</v>
+      </c>
+      <c r="I149" t="n">
+        <v>62</v>
+      </c>
+      <c r="J149" t="n">
+        <v>9</v>
+      </c>
+      <c r="K149" t="n">
+        <v>1794</v>
+      </c>
+      <c r="L149" t="n">
+        <v>10</v>
+      </c>
+      <c r="M149" t="s">
+        <v>253</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-21]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="257">
   <si>
     <t>date</t>
   </si>
@@ -783,6 +783,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/finland/ykkosliiga/, /football/ireland/division-1/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">546dc5f5f7eef1983e54dd54659595ceb263a715</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/pershaya-liga/, /football/ireland/division-1/, /football/malawi/super-league/, /football/mexico/liga-mx/, /football/norway/obos-ligaen/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -7238,6 +7244,47 @@
         <v>255</v>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" s="1" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B151" t="s">
+        <v>256</v>
+      </c>
+      <c r="C151" t="s">
+        <v>31</v>
+      </c>
+      <c r="D151" t="n">
+        <v>136.14340304931</v>
+      </c>
+      <c r="E151" t="n">
+        <v>20</v>
+      </c>
+      <c r="F151" t="n">
+        <v>0</v>
+      </c>
+      <c r="G151" t="n">
+        <v>103</v>
+      </c>
+      <c r="H151" t="n">
+        <v>37</v>
+      </c>
+      <c r="I151" t="n">
+        <v>66</v>
+      </c>
+      <c r="J151" t="n">
+        <v>10</v>
+      </c>
+      <c r="K151" t="n">
+        <v>1823</v>
+      </c>
+      <c r="L151" t="n">
+        <v>10</v>
+      </c>
+      <c r="M151" t="s">
+        <v>257</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-22]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="261">
   <si>
     <t>date</t>
   </si>
@@ -795,6 +795,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/australia/npl-northern-nsw/, /football/estonia/esiliiga/, /football/finland/veikkausliiga/, /football/ireland/premier-division/, /football/ireland/division-1/, /football/norway/obos-ligaen/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">98305fc7f2d6fa067ab120bfcc1699a984600630</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/iceland/besta-deild-karla/, /football/iceland/division-1/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/mexico/liga-mx/, /football/norway/obos-ligaen/, /football/sweden/superettan/</t>
   </si>
 </sst>
 </file>
@@ -7332,6 +7338,47 @@
         <v>259</v>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B153" t="s">
+        <v>260</v>
+      </c>
+      <c r="C153" t="s">
+        <v>31</v>
+      </c>
+      <c r="D153" t="n">
+        <v>176.496753076712</v>
+      </c>
+      <c r="E153" t="n">
+        <v>10</v>
+      </c>
+      <c r="F153" t="n">
+        <v>0</v>
+      </c>
+      <c r="G153" t="n">
+        <v>42</v>
+      </c>
+      <c r="H153" t="n">
+        <v>16</v>
+      </c>
+      <c r="I153" t="n">
+        <v>26</v>
+      </c>
+      <c r="J153" t="n">
+        <v>0</v>
+      </c>
+      <c r="K153" t="n">
+        <v>926</v>
+      </c>
+      <c r="L153" t="n">
+        <v>2</v>
+      </c>
+      <c r="M153" t="s">
+        <v>261</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-23]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="265">
   <si>
     <t>date</t>
   </si>
@@ -807,6 +807,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/ethiopia/premier-league/, /football/finland/ykkosliiga/, /football/ireland/premier-division/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ef0df3898bb43edac0271a92d84f552ef36f5804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/iceland/division-1/, /football/ireland/premier-division/, /football/kazakhstan/premier-league/, /football/lithuania/i-lyga/, /football/mexico/liga-mx/</t>
   </si>
 </sst>
 </file>
@@ -7426,6 +7432,47 @@
         <v>263</v>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" s="1" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B155" t="s">
+        <v>264</v>
+      </c>
+      <c r="C155" t="s">
+        <v>31</v>
+      </c>
+      <c r="D155" t="n">
+        <v>120.377521630128</v>
+      </c>
+      <c r="E155" t="n">
+        <v>12</v>
+      </c>
+      <c r="F155" t="n">
+        <v>0</v>
+      </c>
+      <c r="G155" t="n">
+        <v>62</v>
+      </c>
+      <c r="H155" t="n">
+        <v>24</v>
+      </c>
+      <c r="I155" t="n">
+        <v>38</v>
+      </c>
+      <c r="J155" t="n">
+        <v>12</v>
+      </c>
+      <c r="K155" t="n">
+        <v>1206</v>
+      </c>
+      <c r="L155" t="n">
+        <v>4</v>
+      </c>
+      <c r="M155" t="s">
+        <v>265</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-24]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="269">
   <si>
     <t>date</t>
   </si>
@@ -819,6 +819,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b2eff524f372d74f063e2c84c0527fad30da0ca1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/iceland/division-1/, /football/ireland/premier-division/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/</t>
   </si>
 </sst>
 </file>
@@ -7520,6 +7526,47 @@
         <v>267</v>
       </c>
     </row>
+    <row r="157">
+      <c r="A157" s="1" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B157" t="s">
+        <v>268</v>
+      </c>
+      <c r="C157" t="s">
+        <v>31</v>
+      </c>
+      <c r="D157" t="n">
+        <v>79.4401571551959</v>
+      </c>
+      <c r="E157" t="n">
+        <v>12</v>
+      </c>
+      <c r="F157" t="n">
+        <v>0</v>
+      </c>
+      <c r="G157" t="n">
+        <v>66</v>
+      </c>
+      <c r="H157" t="n">
+        <v>10</v>
+      </c>
+      <c r="I157" t="n">
+        <v>56</v>
+      </c>
+      <c r="J157" t="n">
+        <v>4</v>
+      </c>
+      <c r="K157" t="n">
+        <v>1159</v>
+      </c>
+      <c r="L157" t="n">
+        <v>4</v>
+      </c>
+      <c r="M157" t="s">
+        <v>269</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-25]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="273">
   <si>
     <t>date</t>
   </si>
@@ -831,6 +831,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/finland/ykkosliiga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32a3e54cb2f8538827b3bc9d47e1742e260483c9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/estonia/meistriliiga/, /football/finland/ykkosliiga/, /football/paraguay/division-intermedia/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -7614,6 +7620,47 @@
         <v>271</v>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" s="1" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B159" t="s">
+        <v>272</v>
+      </c>
+      <c r="C159" t="s">
+        <v>31</v>
+      </c>
+      <c r="D159" t="n">
+        <v>120.231960237026</v>
+      </c>
+      <c r="E159" t="n">
+        <v>17</v>
+      </c>
+      <c r="F159" t="n">
+        <v>0</v>
+      </c>
+      <c r="G159" t="n">
+        <v>91</v>
+      </c>
+      <c r="H159" t="n">
+        <v>40</v>
+      </c>
+      <c r="I159" t="n">
+        <v>51</v>
+      </c>
+      <c r="J159" t="n">
+        <v>3</v>
+      </c>
+      <c r="K159" t="n">
+        <v>1367</v>
+      </c>
+      <c r="L159" t="n">
+        <v>10</v>
+      </c>
+      <c r="M159" t="s">
+        <v>273</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-26]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="277">
   <si>
     <t>date</t>
   </si>
@@ -843,6 +843,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/meistriliiga/, /football/ethiopia/premier-league/, /football/finland/veikkausliiga/, /football/finland/ykkosliiga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0b55ffd86bcc73321df4400cad4c7f48c99e1aaf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/ethiopia/premier-league/, /football/faroe-islands/premier-league/, /football/finland/ykkosliiga/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -7708,6 +7714,47 @@
         <v>275</v>
       </c>
     </row>
+    <row r="161">
+      <c r="A161" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B161" t="s">
+        <v>276</v>
+      </c>
+      <c r="C161" t="s">
+        <v>31</v>
+      </c>
+      <c r="D161" t="n">
+        <v>114.748370651404</v>
+      </c>
+      <c r="E161" t="n">
+        <v>21</v>
+      </c>
+      <c r="F161" t="n">
+        <v>0</v>
+      </c>
+      <c r="G161" t="n">
+        <v>126</v>
+      </c>
+      <c r="H161" t="n">
+        <v>69</v>
+      </c>
+      <c r="I161" t="n">
+        <v>57</v>
+      </c>
+      <c r="J161" t="n">
+        <v>1</v>
+      </c>
+      <c r="K161" t="n">
+        <v>1795</v>
+      </c>
+      <c r="L161" t="n">
+        <v>12</v>
+      </c>
+      <c r="M161" t="s">
+        <v>277</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-27]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="281">
   <si>
     <t>date</t>
   </si>
@@ -855,6 +855,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/finland/ykkosliiga/, /football/iceland/besta-deild-karla/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e365b84d4b4609d4a74be26f45543daacae4f0a7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/ethiopia/premier-league/, /football/faroe-islands/premier-league/, /football/ireland/premier-division/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -7802,6 +7808,47 @@
         <v>279</v>
       </c>
     </row>
+    <row r="163">
+      <c r="A163" s="1" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B163" t="s">
+        <v>280</v>
+      </c>
+      <c r="C163" t="s">
+        <v>31</v>
+      </c>
+      <c r="D163" t="n">
+        <v>108.437464487553</v>
+      </c>
+      <c r="E163" t="n">
+        <v>26</v>
+      </c>
+      <c r="F163" t="n">
+        <v>0</v>
+      </c>
+      <c r="G163" t="n">
+        <v>125</v>
+      </c>
+      <c r="H163" t="n">
+        <v>72</v>
+      </c>
+      <c r="I163" t="n">
+        <v>53</v>
+      </c>
+      <c r="J163" t="n">
+        <v>9</v>
+      </c>
+      <c r="K163" t="n">
+        <v>2121</v>
+      </c>
+      <c r="L163" t="n">
+        <v>13</v>
+      </c>
+      <c r="M163" t="s">
+        <v>281</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-28]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="285">
   <si>
     <t>date</t>
   </si>
@@ -867,6 +867,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/faroe-islands/premier-league/, /football/finland/veikkausliiga/, /football/ireland/premier-division/, /football/norway/obos-ligaen/, /football/peru/liga-1/, /football/south-korea/k-league-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">978cc95cc3a654d122ff2fae60feddbd7896e424</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/ireland/premier-division/, /football/norway/obos-ligaen/, /football/paraguay/division-intermedia/, /football/south-korea/k-league-2/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -7896,6 +7902,47 @@
         <v>283</v>
       </c>
     </row>
+    <row r="165">
+      <c r="A165" s="1" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B165" t="s">
+        <v>284</v>
+      </c>
+      <c r="C165" t="s">
+        <v>31</v>
+      </c>
+      <c r="D165" t="n">
+        <v>118.674274476369</v>
+      </c>
+      <c r="E165" t="n">
+        <v>21</v>
+      </c>
+      <c r="F165" t="n">
+        <v>0</v>
+      </c>
+      <c r="G165" t="n">
+        <v>93</v>
+      </c>
+      <c r="H165" t="n">
+        <v>53</v>
+      </c>
+      <c r="I165" t="n">
+        <v>40</v>
+      </c>
+      <c r="J165" t="n">
+        <v>9</v>
+      </c>
+      <c r="K165" t="n">
+        <v>1781</v>
+      </c>
+      <c r="L165" t="n">
+        <v>12</v>
+      </c>
+      <c r="M165" t="s">
+        <v>285</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-29]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="289">
   <si>
     <t>date</t>
   </si>
@@ -879,6 +879,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/meistriliiga/, /football/ethiopia/premier-league/, /football/finland/veikkausliiga/, /football/iceland/besta-deild-karla/, /football/mexico/liga-mx/, /football/norway/eliteserien/, /football/norway/obos-ligaen/, /football/peru/liga-1/, /football/scotland/premiership/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">720abf67e4ab168f8c5913c786f70e6f7d126ad8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/faroe-islands/premier-league/, /football/finland/ykkosliiga/, /football/iceland/division-1/, /football/ireland/division-1/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/peru/liga-1/, /football/romania/superliga/</t>
   </si>
 </sst>
 </file>
@@ -7990,6 +7996,47 @@
         <v>287</v>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" s="1" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B167" t="s">
+        <v>288</v>
+      </c>
+      <c r="C167" t="s">
+        <v>31</v>
+      </c>
+      <c r="D167" t="n">
+        <v>123.079222019513</v>
+      </c>
+      <c r="E167" t="n">
+        <v>17</v>
+      </c>
+      <c r="F167" t="n">
+        <v>0</v>
+      </c>
+      <c r="G167" t="n">
+        <v>96</v>
+      </c>
+      <c r="H167" t="n">
+        <v>41</v>
+      </c>
+      <c r="I167" t="n">
+        <v>55</v>
+      </c>
+      <c r="J167" t="n">
+        <v>5</v>
+      </c>
+      <c r="K167" t="n">
+        <v>1830</v>
+      </c>
+      <c r="L167" t="n">
+        <v>6</v>
+      </c>
+      <c r="M167" t="s">
+        <v>289</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-06-30]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="291">
   <si>
     <t>date</t>
   </si>
@@ -885,6 +885,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/faroe-islands/premier-league/, /football/finland/ykkosliiga/, /football/iceland/division-1/, /football/ireland/division-1/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/peru/liga-1/, /football/romania/superliga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bc1b28bbee95c80bba7288595410f8a45a5300fc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/bundesliga/, /football/belarus/vysshaya-liga/, /football/ethiopia/premier-league/, /football/iceland/division-1/, /football/ireland/division-1/, /football/kazakhstan/premier-league/, /football/lithuania/i-lyga/, /football/mexico/liga-mx/, /football/peru/liga-1/</t>
   </si>
 </sst>
 </file>
@@ -8037,6 +8043,47 @@
         <v>289</v>
       </c>
     </row>
+    <row r="168">
+      <c r="A168" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B168" t="s">
+        <v>290</v>
+      </c>
+      <c r="C168" t="s">
+        <v>31</v>
+      </c>
+      <c r="D168" t="n">
+        <v>162.802585577965</v>
+      </c>
+      <c r="E168" t="n">
+        <v>16</v>
+      </c>
+      <c r="F168" t="n">
+        <v>0</v>
+      </c>
+      <c r="G168" t="n">
+        <v>100</v>
+      </c>
+      <c r="H168" t="n">
+        <v>36</v>
+      </c>
+      <c r="I168" t="n">
+        <v>64</v>
+      </c>
+      <c r="J168" t="n">
+        <v>2</v>
+      </c>
+      <c r="K168" t="n">
+        <v>1820</v>
+      </c>
+      <c r="L168" t="n">
+        <v>8</v>
+      </c>
+      <c r="M168" t="s">
+        <v>291</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-01]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="295">
   <si>
     <t>date</t>
   </si>
@@ -897,6 +897,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/ecuador/serie-b/, /football/romania/superliga/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3dc078ecd8b1c9a70eae2a47967beef7dce03752</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/australia/npl-act/, /football/canada/canadian-premier-league/, /football/finland/ykkosliiga/, /football/iceland/division-1/, /football/ireland/premier-division/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -8131,6 +8137,47 @@
         <v>293</v>
       </c>
     </row>
+    <row r="170">
+      <c r="A170" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B170" t="s">
+        <v>294</v>
+      </c>
+      <c r="C170" t="s">
+        <v>31</v>
+      </c>
+      <c r="D170" t="n">
+        <v>124.06937876145</v>
+      </c>
+      <c r="E170" t="n">
+        <v>22</v>
+      </c>
+      <c r="F170" t="n">
+        <v>0</v>
+      </c>
+      <c r="G170" t="n">
+        <v>116</v>
+      </c>
+      <c r="H170" t="n">
+        <v>53</v>
+      </c>
+      <c r="I170" t="n">
+        <v>63</v>
+      </c>
+      <c r="J170" t="n">
+        <v>1</v>
+      </c>
+      <c r="K170" t="n">
+        <v>2292</v>
+      </c>
+      <c r="L170" t="n">
+        <v>12</v>
+      </c>
+      <c r="M170" t="s">
+        <v>295</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-02]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="297">
   <si>
     <t>date</t>
   </si>
@@ -903,6 +903,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/australia/npl-act/, /football/canada/canadian-premier-league/, /football/finland/ykkosliiga/, /football/iceland/division-1/, /football/ireland/premier-division/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0d502cabbbf7b11aa78d8b88a195ef0c2f0928f6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/canada/canadian-premier-league/, /football/finland/ykkosliiga/, /football/mexico/liga-mx/, /football/romania/superliga/, /football/uruguay/segunda-division/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -8178,6 +8184,47 @@
         <v>295</v>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" s="1" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B171" t="s">
+        <v>296</v>
+      </c>
+      <c r="C171" t="s">
+        <v>31</v>
+      </c>
+      <c r="D171" t="n">
+        <v>158.929395572344</v>
+      </c>
+      <c r="E171" t="n">
+        <v>26</v>
+      </c>
+      <c r="F171" t="n">
+        <v>0</v>
+      </c>
+      <c r="G171" t="n">
+        <v>132</v>
+      </c>
+      <c r="H171" t="n">
+        <v>67</v>
+      </c>
+      <c r="I171" t="n">
+        <v>65</v>
+      </c>
+      <c r="J171" t="n">
+        <v>2</v>
+      </c>
+      <c r="K171" t="n">
+        <v>2438</v>
+      </c>
+      <c r="L171" t="n">
+        <v>15</v>
+      </c>
+      <c r="M171" t="s">
+        <v>297</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-03]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="299">
   <si>
     <t>date</t>
   </si>
@@ -909,6 +909,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/canada/canadian-premier-league/, /football/finland/ykkosliiga/, /football/mexico/liga-mx/, /football/romania/superliga/, /football/uruguay/segunda-division/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">88f171f070cf47c692b6092cf9ce6877dbf8e148</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/estonia/meistriliiga/, /football/estonia/esiliiga/, /football/ethiopia/premier-league/, /football/kazakhstan/premier-league/, /football/paraguay/division-intermedia/, /football/romania/superliga/</t>
   </si>
 </sst>
 </file>
@@ -8225,6 +8231,47 @@
         <v>297</v>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B172" t="s">
+        <v>298</v>
+      </c>
+      <c r="C172" t="s">
+        <v>31</v>
+      </c>
+      <c r="D172" t="n">
+        <v>130.789730147521</v>
+      </c>
+      <c r="E172" t="n">
+        <v>29</v>
+      </c>
+      <c r="F172" t="n">
+        <v>0</v>
+      </c>
+      <c r="G172" t="n">
+        <v>155</v>
+      </c>
+      <c r="H172" t="n">
+        <v>82</v>
+      </c>
+      <c r="I172" t="n">
+        <v>73</v>
+      </c>
+      <c r="J172" t="n">
+        <v>4</v>
+      </c>
+      <c r="K172" t="n">
+        <v>2599</v>
+      </c>
+      <c r="L172" t="n">
+        <v>18</v>
+      </c>
+      <c r="M172" t="s">
+        <v>299</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-04]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="303">
   <si>
     <t>date</t>
   </si>
@@ -921,6 +921,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/meistriliiga/, /football/paraguay/division-intermedia/, /football/peru/liga-1/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">287ee871cdc0fc3802e6599a4a1a74fb0e89f4ed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/estonia/meistriliiga/, /football/germany/2-bundesliga/, /football/peru/liga-1/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -8319,6 +8325,47 @@
         <v>301</v>
       </c>
     </row>
+    <row r="174">
+      <c r="A174" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B174" t="s">
+        <v>302</v>
+      </c>
+      <c r="C174" t="s">
+        <v>31</v>
+      </c>
+      <c r="D174" t="n">
+        <v>138.986416443189</v>
+      </c>
+      <c r="E174" t="n">
+        <v>24</v>
+      </c>
+      <c r="F174" t="n">
+        <v>0</v>
+      </c>
+      <c r="G174" t="n">
+        <v>106</v>
+      </c>
+      <c r="H174" t="n">
+        <v>69</v>
+      </c>
+      <c r="I174" t="n">
+        <v>37</v>
+      </c>
+      <c r="J174" t="n">
+        <v>10</v>
+      </c>
+      <c r="K174" t="n">
+        <v>1893</v>
+      </c>
+      <c r="L174" t="n">
+        <v>14</v>
+      </c>
+      <c r="M174" t="s">
+        <v>303</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-05]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="307">
   <si>
     <t>date</t>
   </si>
@@ -933,6 +933,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/finland/veikkausliiga/, /football/finland/ykkosliiga/, /football/ireland/division-1/, /football/paraguay/division-intermedia/, /football/romania/superliga/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6d381387afcbe10fffaa6a141923beeb86375d72</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/finland/veikkausliiga/, /football/finland/veikkausliiga/, /football/finland/ykkosliiga/, /football/ireland/division-1/, /football/malawi/super-league/, /football/romania/superliga/, /football/scotland/premiership/</t>
   </si>
 </sst>
 </file>
@@ -8413,6 +8419,47 @@
         <v>305</v>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" s="1" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B176" t="s">
+        <v>306</v>
+      </c>
+      <c r="C176" t="s">
+        <v>31</v>
+      </c>
+      <c r="D176" t="n">
+        <v>116.446991058191</v>
+      </c>
+      <c r="E176" t="n">
+        <v>31</v>
+      </c>
+      <c r="F176" t="n">
+        <v>0</v>
+      </c>
+      <c r="G176" t="n">
+        <v>110</v>
+      </c>
+      <c r="H176" t="n">
+        <v>47</v>
+      </c>
+      <c r="I176" t="n">
+        <v>63</v>
+      </c>
+      <c r="J176" t="n">
+        <v>14</v>
+      </c>
+      <c r="K176" t="n">
+        <v>2894</v>
+      </c>
+      <c r="L176" t="n">
+        <v>15</v>
+      </c>
+      <c r="M176" t="s">
+        <v>307</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-06]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="311">
   <si>
     <t>date</t>
   </si>
@@ -945,6 +945,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/canada/canadian-premier-league/, /football/estonia/meistriliiga/, /football/finland/ykkosliiga/, /football/peru/liga-1/, /football/romania/superliga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e4168081185ce76c72e477d39dbdfb4ea7606893</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/australia/npl-northern-nsw/, /football/canada/canadian-premier-league/, /football/estonia/meistriliiga/, /football/ireland/division-1/</t>
   </si>
 </sst>
 </file>
@@ -8507,6 +8513,47 @@
         <v>309</v>
       </c>
     </row>
+    <row r="178">
+      <c r="A178" s="1" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B178" t="s">
+        <v>310</v>
+      </c>
+      <c r="C178" t="s">
+        <v>31</v>
+      </c>
+      <c r="D178" t="n">
+        <v>84.0726300875346</v>
+      </c>
+      <c r="E178" t="n">
+        <v>21</v>
+      </c>
+      <c r="F178" t="n">
+        <v>0</v>
+      </c>
+      <c r="G178" t="n">
+        <v>110</v>
+      </c>
+      <c r="H178" t="n">
+        <v>44</v>
+      </c>
+      <c r="I178" t="n">
+        <v>66</v>
+      </c>
+      <c r="J178" t="n">
+        <v>15</v>
+      </c>
+      <c r="K178" t="n">
+        <v>2184</v>
+      </c>
+      <c r="L178" t="n">
+        <v>7</v>
+      </c>
+      <c r="M178" t="s">
+        <v>311</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-07]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="315">
   <si>
     <t>date</t>
   </si>
@@ -957,6 +957,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/canada/canadian-premier-league/, /football/iceland/division-1/, /football/kazakhstan/premier-league/, /football/romania/superliga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b2abc40c10f421a9a5a8308946f52ccd3e6c0dac</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/argentina/primera-nacional/, /football/australia/npl-northern-nsw/, /football/finland/ykkosliiga/, /football/germany/2-bundesliga/, /football/iceland/besta-deild-karla/, /football/iceland/division-1/</t>
   </si>
 </sst>
 </file>
@@ -8601,6 +8607,47 @@
         <v>313</v>
       </c>
     </row>
+    <row r="180">
+      <c r="A180" s="1" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B180" t="s">
+        <v>314</v>
+      </c>
+      <c r="C180" t="s">
+        <v>31</v>
+      </c>
+      <c r="D180" t="n">
+        <v>126.921021250884</v>
+      </c>
+      <c r="E180" t="n">
+        <v>22</v>
+      </c>
+      <c r="F180" t="n">
+        <v>0</v>
+      </c>
+      <c r="G180" t="n">
+        <v>107</v>
+      </c>
+      <c r="H180" t="n">
+        <v>28</v>
+      </c>
+      <c r="I180" t="n">
+        <v>79</v>
+      </c>
+      <c r="J180" t="n">
+        <v>3</v>
+      </c>
+      <c r="K180" t="n">
+        <v>2294</v>
+      </c>
+      <c r="L180" t="n">
+        <v>7</v>
+      </c>
+      <c r="M180" t="s">
+        <v>315</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-08]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="319">
   <si>
     <t>date</t>
   </si>
@@ -969,6 +969,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/argentina/primera-nacional/, /football/australia/npl-northern-nsw/, /football/austria/bundesliga/, /football/belarus/vysshaya-liga/, /football/bolivia/division-profesional/, /football/iceland/besta-deild-karla/, /football/kazakhstan/premier-league/, /football/mexico/liga-mx/, /football/peru/liga-1/, /football/romania/superliga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">537a5a46ea6344a2b10c2099e37b52ac717f8214</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/australia/npl-act/, /football/belarus/vysshaya-liga/, /football/canada/canadian-premier-league/, /football/finland/ykkosliiga/, /football/iceland/besta-deild-karla/, /football/iceland/division-1/, /football/ireland/division-1/</t>
   </si>
 </sst>
 </file>
@@ -8695,6 +8701,47 @@
         <v>317</v>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" s="1" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B182" t="s">
+        <v>318</v>
+      </c>
+      <c r="C182" t="s">
+        <v>31</v>
+      </c>
+      <c r="D182" t="n">
+        <v>122.87478047212</v>
+      </c>
+      <c r="E182" t="n">
+        <v>23</v>
+      </c>
+      <c r="F182" t="n">
+        <v>0</v>
+      </c>
+      <c r="G182" t="n">
+        <v>136</v>
+      </c>
+      <c r="H182" t="n">
+        <v>50</v>
+      </c>
+      <c r="I182" t="n">
+        <v>86</v>
+      </c>
+      <c r="J182" t="n">
+        <v>2</v>
+      </c>
+      <c r="K182" t="n">
+        <v>2637</v>
+      </c>
+      <c r="L182" t="n">
+        <v>8</v>
+      </c>
+      <c r="M182" t="s">
+        <v>319</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-09]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="323">
   <si>
     <t>date</t>
   </si>
@@ -981,6 +981,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/canada/canadian-premier-league/, /football/finland/ykkosliiga/, /football/kazakhstan/premier-league/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1fd3157269f813f98d3f458cb7e42513e88d3f41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/peru/liga-1/, /football/uruguay/segunda-division/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -8789,6 +8795,47 @@
         <v>321</v>
       </c>
     </row>
+    <row r="184">
+      <c r="A184" s="1" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B184" t="s">
+        <v>322</v>
+      </c>
+      <c r="C184" t="s">
+        <v>31</v>
+      </c>
+      <c r="D184" t="n">
+        <v>101.856391445796</v>
+      </c>
+      <c r="E184" t="n">
+        <v>28</v>
+      </c>
+      <c r="F184" t="n">
+        <v>0</v>
+      </c>
+      <c r="G184" t="n">
+        <v>153</v>
+      </c>
+      <c r="H184" t="n">
+        <v>63</v>
+      </c>
+      <c r="I184" t="n">
+        <v>90</v>
+      </c>
+      <c r="J184" t="n">
+        <v>3</v>
+      </c>
+      <c r="K184" t="n">
+        <v>2700</v>
+      </c>
+      <c r="L184" t="n">
+        <v>14</v>
+      </c>
+      <c r="M184" t="s">
+        <v>323</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-10]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="327">
   <si>
     <t>date</t>
   </si>
@@ -993,6 +993,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/esiliiga/, /football/kazakhstan/premier-league/, /football/poland/ekstraklasa/, /football/romania/superliga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7d0c05b90fd0e286db40bc780de7109e6da06e7b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/finland/ykkosliiga/, /football/paraguay/division-intermedia/, /football/poland/ekstraklasa/, /football/romania/superliga/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -8883,6 +8889,47 @@
         <v>325</v>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B186" t="s">
+        <v>326</v>
+      </c>
+      <c r="C186" t="s">
+        <v>31</v>
+      </c>
+      <c r="D186" t="n">
+        <v>134.705934043725</v>
+      </c>
+      <c r="E186" t="n">
+        <v>28</v>
+      </c>
+      <c r="F186" t="n">
+        <v>0</v>
+      </c>
+      <c r="G186" t="n">
+        <v>178</v>
+      </c>
+      <c r="H186" t="n">
+        <v>81</v>
+      </c>
+      <c r="I186" t="n">
+        <v>97</v>
+      </c>
+      <c r="J186" t="n">
+        <v>1</v>
+      </c>
+      <c r="K186" t="n">
+        <v>2809</v>
+      </c>
+      <c r="L186" t="n">
+        <v>14</v>
+      </c>
+      <c r="M186" t="s">
+        <v>327</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-11]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="331">
   <si>
     <t>date</t>
   </si>
@@ -1005,6 +1005,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/canada/canadian-premier-league/, /football/paraguay/division-intermedia/, /football/peru/liga-1/, /football/romania/superliga/, /football/scotland/premiership/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2e94cec98a4c301f35aa5a3160d14b0a0ff56be6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/australia/npl-act/, /football/belarus/pershaya-liga/, /football/colombia/primera-a/, /football/paraguay/division-intermedia/, /football/uruguay/segunda-division/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -8977,6 +8983,47 @@
         <v>329</v>
       </c>
     </row>
+    <row r="188">
+      <c r="A188" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B188" t="s">
+        <v>330</v>
+      </c>
+      <c r="C188" t="s">
+        <v>31</v>
+      </c>
+      <c r="D188" t="n">
+        <v>130.042080553373</v>
+      </c>
+      <c r="E188" t="n">
+        <v>37</v>
+      </c>
+      <c r="F188" t="n">
+        <v>0</v>
+      </c>
+      <c r="G188" t="n">
+        <v>173</v>
+      </c>
+      <c r="H188" t="n">
+        <v>72</v>
+      </c>
+      <c r="I188" t="n">
+        <v>101</v>
+      </c>
+      <c r="J188" t="n">
+        <v>5</v>
+      </c>
+      <c r="K188" t="n">
+        <v>3230</v>
+      </c>
+      <c r="L188" t="n">
+        <v>13</v>
+      </c>
+      <c r="M188" t="s">
+        <v>331</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-12]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="335">
   <si>
     <t>date</t>
   </si>
@@ -1017,6 +1017,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/china/super-league/, /football/estonia/esiliiga/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ec8718c6d5c533311e78e9843d471414d704b40c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/ecuador/serie-b/, /football/finland/veikkausliiga/, /football/iceland/besta-deild-karla/, /football/peru/liga-1/, /football/romania/superliga/, /football/south-korea/k-league-2/, /football/south-korea/k-league-2/</t>
   </si>
 </sst>
 </file>
@@ -9071,6 +9077,47 @@
         <v>333</v>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" s="1" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B190" t="s">
+        <v>334</v>
+      </c>
+      <c r="C190" t="s">
+        <v>31</v>
+      </c>
+      <c r="D190" t="n">
+        <v>149.13395550251</v>
+      </c>
+      <c r="E190" t="n">
+        <v>23</v>
+      </c>
+      <c r="F190" t="n">
+        <v>0</v>
+      </c>
+      <c r="G190" t="n">
+        <v>122</v>
+      </c>
+      <c r="H190" t="n">
+        <v>45</v>
+      </c>
+      <c r="I190" t="n">
+        <v>77</v>
+      </c>
+      <c r="J190" t="n">
+        <v>33</v>
+      </c>
+      <c r="K190" t="n">
+        <v>2363</v>
+      </c>
+      <c r="L190" t="n">
+        <v>7</v>
+      </c>
+      <c r="M190" t="s">
+        <v>335</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-13]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="337">
   <si>
     <t>date</t>
   </si>
@@ -1023,6 +1023,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/ecuador/serie-b/, /football/finland/veikkausliiga/, /football/iceland/besta-deild-karla/, /football/peru/liga-1/, /football/romania/superliga/, /football/south-korea/k-league-2/, /football/south-korea/k-league-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c8be516f8e59b57510d908a165a33b8bf32903d1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/croatia/hnl/, /football/denmark/superliga/, /football/peru/liga-1/, /football/romania/superliga/</t>
   </si>
 </sst>
 </file>
@@ -9118,6 +9124,47 @@
         <v>335</v>
       </c>
     </row>
+    <row r="191">
+      <c r="A191" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B191" t="s">
+        <v>336</v>
+      </c>
+      <c r="C191" t="s">
+        <v>31</v>
+      </c>
+      <c r="D191" t="n">
+        <v>150.716102230549</v>
+      </c>
+      <c r="E191" t="n">
+        <v>26</v>
+      </c>
+      <c r="F191" t="n">
+        <v>0</v>
+      </c>
+      <c r="G191" t="n">
+        <v>174</v>
+      </c>
+      <c r="H191" t="n">
+        <v>101</v>
+      </c>
+      <c r="I191" t="n">
+        <v>73</v>
+      </c>
+      <c r="J191" t="n">
+        <v>20</v>
+      </c>
+      <c r="K191" t="n">
+        <v>2950</v>
+      </c>
+      <c r="L191" t="n">
+        <v>13</v>
+      </c>
+      <c r="M191" t="s">
+        <v>337</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-14]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="341">
   <si>
     <t>date</t>
   </si>
@@ -1035,6 +1035,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/meistriliiga/, /football/finland/ykkosliiga/, /football/iceland/division-1/, /football/kazakhstan/premier-league/, /football/peru/liga-1/, /football/uruguay/segunda-division/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">313f93ca3b4282dd0de7e9005afff78c7f5b24fb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/australia/npl-northern-nsw/, /football/canada/canadian-premier-league/, /football/colombia/primera-a/, /football/ecuador/serie-b/, /football/iceland/division-1/, /football/kazakhstan/premier-league/, /football/peru/liga-1/, /football/poland/ekstraklasa/, /football/romania/superliga/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -9212,6 +9218,47 @@
         <v>339</v>
       </c>
     </row>
+    <row r="193">
+      <c r="A193" s="1" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B193" t="s">
+        <v>340</v>
+      </c>
+      <c r="C193" t="s">
+        <v>31</v>
+      </c>
+      <c r="D193" t="n">
+        <v>204.831943142414</v>
+      </c>
+      <c r="E193" t="n">
+        <v>25</v>
+      </c>
+      <c r="F193" t="n">
+        <v>0</v>
+      </c>
+      <c r="G193" t="n">
+        <v>183</v>
+      </c>
+      <c r="H193" t="n">
+        <v>71</v>
+      </c>
+      <c r="I193" t="n">
+        <v>112</v>
+      </c>
+      <c r="J193" t="n">
+        <v>3</v>
+      </c>
+      <c r="K193" t="n">
+        <v>2700</v>
+      </c>
+      <c r="L193" t="n">
+        <v>9</v>
+      </c>
+      <c r="M193" t="s">
+        <v>341</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-15]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="345">
   <si>
     <t>date</t>
   </si>
@@ -1047,6 +1047,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/iceland/division-1/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3a8bd97893f570e71a2cfd614757dde235d3c1b5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belgium/jupiler-pro-league/, /football/canada/canadian-premier-league/, /football/colombia/primera-a/, /football/estonia/meistriliiga/, /football/estonia/esiliiga/, /football/iceland/division-1/, /football/lithuania/i-lyga/, /football/peru/liga-1/, /football/uzbekistan/super-league/</t>
   </si>
 </sst>
 </file>
@@ -9306,6 +9312,47 @@
         <v>343</v>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B195" t="s">
+        <v>344</v>
+      </c>
+      <c r="C195" t="s">
+        <v>31</v>
+      </c>
+      <c r="D195" t="n">
+        <v>183.366394817829</v>
+      </c>
+      <c r="E195" t="n">
+        <v>32</v>
+      </c>
+      <c r="F195" t="n">
+        <v>0</v>
+      </c>
+      <c r="G195" t="n">
+        <v>201</v>
+      </c>
+      <c r="H195" t="n">
+        <v>81</v>
+      </c>
+      <c r="I195" t="n">
+        <v>120</v>
+      </c>
+      <c r="J195" t="n">
+        <v>3</v>
+      </c>
+      <c r="K195" t="n">
+        <v>3373</v>
+      </c>
+      <c r="L195" t="n">
+        <v>14</v>
+      </c>
+      <c r="M195" t="s">
+        <v>345</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-16]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="349">
   <si>
     <t>date</t>
   </si>
@@ -1059,6 +1059,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/esiliiga/, /football/latvia/virsliga/, /football/poland/ekstraklasa/, /football/romania/superliga/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3719f9821e6caa50b0ef633215165ed1bfc3517d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/chile/liga-de-ascenso/, /football/chile/liga-de-ascenso/, /football/colombia/primera-a/, /football/lithuania/i-lyga/, /football/poland/ekstraklasa/, /football/uruguay/segunda-division/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -9400,6 +9406,47 @@
         <v>347</v>
       </c>
     </row>
+    <row r="197">
+      <c r="A197" s="1" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B197" t="s">
+        <v>348</v>
+      </c>
+      <c r="C197" t="s">
+        <v>31</v>
+      </c>
+      <c r="D197" t="n">
+        <v>231.644274826845</v>
+      </c>
+      <c r="E197" t="n">
+        <v>34</v>
+      </c>
+      <c r="F197" t="n">
+        <v>0</v>
+      </c>
+      <c r="G197" t="n">
+        <v>226</v>
+      </c>
+      <c r="H197" t="n">
+        <v>85</v>
+      </c>
+      <c r="I197" t="n">
+        <v>141</v>
+      </c>
+      <c r="J197" t="n">
+        <v>2</v>
+      </c>
+      <c r="K197" t="n">
+        <v>3266</v>
+      </c>
+      <c r="L197" t="n">
+        <v>13</v>
+      </c>
+      <c r="M197" t="s">
+        <v>349</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-17]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="351">
   <si>
     <t>date</t>
   </si>
@@ -1065,6 +1065,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/chile/liga-de-ascenso/, /football/chile/liga-de-ascenso/, /football/colombia/primera-a/, /football/lithuania/i-lyga/, /football/poland/ekstraklasa/, /football/uruguay/segunda-division/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b30f4bdc4e5313656632ce13b3102e668ca992f4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belgium/jupiler-pro-league/, /football/bolivia/division-profesional/, /football/colombia/primera-a/, /football/estonia/esiliiga/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -9447,6 +9453,47 @@
         <v>349</v>
       </c>
     </row>
+    <row r="198">
+      <c r="A198" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B198" t="s">
+        <v>350</v>
+      </c>
+      <c r="C198" t="s">
+        <v>31</v>
+      </c>
+      <c r="D198" t="n">
+        <v>184.560771099726</v>
+      </c>
+      <c r="E198" t="n">
+        <v>35</v>
+      </c>
+      <c r="F198" t="n">
+        <v>0</v>
+      </c>
+      <c r="G198" t="n">
+        <v>230</v>
+      </c>
+      <c r="H198" t="n">
+        <v>85</v>
+      </c>
+      <c r="I198" t="n">
+        <v>145</v>
+      </c>
+      <c r="J198" t="n">
+        <v>6</v>
+      </c>
+      <c r="K198" t="n">
+        <v>3449</v>
+      </c>
+      <c r="L198" t="n">
+        <v>15</v>
+      </c>
+      <c r="M198" t="s">
+        <v>351</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-18]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="355">
   <si>
     <t>date</t>
   </si>
@@ -1077,6 +1077,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/latvia/nakotnes-liga/, /football/poland/ekstraklasa/, /football/romania/superliga/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">224875ac673174bbeba3557ef2a39f7ea1f50f1e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belgium/jupiler-pro-league/, /football/bolivia/division-profesional/, /football/colombia/primera-a/, /football/denmark/superliga/, /football/estonia/meistriliiga/, /football/ireland/division-1/, /football/lithuania/i-lyga/, /football/paraguay/copa-de-primera/, /football/romania/superliga/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -9541,6 +9547,47 @@
         <v>353</v>
       </c>
     </row>
+    <row r="200">
+      <c r="A200" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B200" t="s">
+        <v>354</v>
+      </c>
+      <c r="C200" t="s">
+        <v>31</v>
+      </c>
+      <c r="D200" t="n">
+        <v>218.485574400425</v>
+      </c>
+      <c r="E200" t="n">
+        <v>43</v>
+      </c>
+      <c r="F200" t="n">
+        <v>0</v>
+      </c>
+      <c r="G200" t="n">
+        <v>228</v>
+      </c>
+      <c r="H200" t="n">
+        <v>88</v>
+      </c>
+      <c r="I200" t="n">
+        <v>140</v>
+      </c>
+      <c r="J200" t="n">
+        <v>25</v>
+      </c>
+      <c r="K200" t="n">
+        <v>3866</v>
+      </c>
+      <c r="L200" t="n">
+        <v>18</v>
+      </c>
+      <c r="M200" t="s">
+        <v>355</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-19]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="359">
   <si>
     <t>date</t>
   </si>
@@ -1089,6 +1089,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belgium/jupiler-pro-league/, /football/bolivia/division-profesional/, /football/colombia/primera-a/, /football/estonia/esiliiga/, /football/ireland/division-1/, /football/moldova/super-liga/, /football/peru/liga-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">98657035d933d5a1e3da39f2a7eeb5491933ddca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belgium/jupiler-pro-league/, /football/colombia/primera-a/, /football/finland/ykkosliiga/, /football/ireland/premier-division/, /football/ireland/division-1/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -9635,6 +9641,47 @@
         <v>357</v>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" s="1" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B202" t="s">
+        <v>358</v>
+      </c>
+      <c r="C202" t="s">
+        <v>31</v>
+      </c>
+      <c r="D202" t="n">
+        <v>230.527141483625</v>
+      </c>
+      <c r="E202" t="n">
+        <v>41</v>
+      </c>
+      <c r="F202" t="n">
+        <v>0</v>
+      </c>
+      <c r="G202" t="n">
+        <v>191</v>
+      </c>
+      <c r="H202" t="n">
+        <v>67</v>
+      </c>
+      <c r="I202" t="n">
+        <v>124</v>
+      </c>
+      <c r="J202" t="n">
+        <v>11</v>
+      </c>
+      <c r="K202" t="n">
+        <v>3671</v>
+      </c>
+      <c r="L202" t="n">
+        <v>16</v>
+      </c>
+      <c r="M202" t="s">
+        <v>359</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-20]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="363">
   <si>
     <t>date</t>
   </si>
@@ -1101,6 +1101,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belgium/jupiler-pro-league/, /football/bolivia/division-profesional/, /football/peru/liga-1/, /football/romania/superliga/, /football/sweden/superettan/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9aa0befbc193e12e5209f8540ac7782536ac2fd9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/ireland/premier-division/, /football/ireland/division-1/, /football/mexico/liga-de-expansion-mx/, /football/paraguay/copa-de-primera/, /football/poland/ekstraklasa/, /football/slovenia/prva-liga/, /football/south-korea/k-league-2/, /football/uruguay/liga-auf-uruguaya/</t>
   </si>
 </sst>
 </file>
@@ -9729,6 +9735,47 @@
         <v>361</v>
       </c>
     </row>
+    <row r="204">
+      <c r="A204" s="1" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B204" t="s">
+        <v>362</v>
+      </c>
+      <c r="C204" t="s">
+        <v>31</v>
+      </c>
+      <c r="D204" t="n">
+        <v>168.277345709006</v>
+      </c>
+      <c r="E204" t="n">
+        <v>31</v>
+      </c>
+      <c r="F204" t="n">
+        <v>0</v>
+      </c>
+      <c r="G204" t="n">
+        <v>193</v>
+      </c>
+      <c r="H204" t="n">
+        <v>42</v>
+      </c>
+      <c r="I204" t="n">
+        <v>151</v>
+      </c>
+      <c r="J204" t="n">
+        <v>6</v>
+      </c>
+      <c r="K204" t="n">
+        <v>3210</v>
+      </c>
+      <c r="L204" t="n">
+        <v>6</v>
+      </c>
+      <c r="M204" t="s">
+        <v>363</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-22]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="365">
   <si>
     <t>date</t>
   </si>
@@ -1107,6 +1107,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/ireland/premier-division/, /football/ireland/division-1/, /football/mexico/liga-de-expansion-mx/, /football/paraguay/copa-de-primera/, /football/poland/ekstraklasa/, /football/slovenia/prva-liga/, /football/south-korea/k-league-2/, /football/uruguay/liga-auf-uruguaya/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d296343bf19c97616acffc8795a9246146d026bf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/bundesliga/, /football/belgium/jupiler-pro-league/, /football/brazil/serie-a-betano/, /football/canada/canadian-premier-league/, /football/estonia/meistriliiga/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/lithuania/i-lyga/, /football/spain/laliga/</t>
   </si>
 </sst>
 </file>
@@ -9776,6 +9782,47 @@
         <v>363</v>
       </c>
     </row>
+    <row r="205">
+      <c r="A205" s="1" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B205" t="s">
+        <v>364</v>
+      </c>
+      <c r="C205" t="s">
+        <v>31</v>
+      </c>
+      <c r="D205" t="n">
+        <v>218.657258208593</v>
+      </c>
+      <c r="E205" t="n">
+        <v>31</v>
+      </c>
+      <c r="F205" t="n">
+        <v>0</v>
+      </c>
+      <c r="G205" t="n">
+        <v>227</v>
+      </c>
+      <c r="H205" t="n">
+        <v>91</v>
+      </c>
+      <c r="I205" t="n">
+        <v>136</v>
+      </c>
+      <c r="J205" t="n">
+        <v>21</v>
+      </c>
+      <c r="K205" t="n">
+        <v>3127</v>
+      </c>
+      <c r="L205" t="n">
+        <v>8</v>
+      </c>
+      <c r="M205" t="s">
+        <v>365</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-23]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="369">
   <si>
     <t>date</t>
   </si>
@@ -1119,6 +1119,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/canada/canadian-premier-league/, /football/estonia/meistriliiga/, /football/finland/ykkosliiga/, /football/iceland/division-1/, /football/romania/superliga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">70cd21e44872c78cb1ab410a2484d05a062017db</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/australia/npl-act/, /football/colombia/primera-a/, /football/croatia/hnl/, /football/estonia/meistriliiga/, /football/finland/ykkosliiga/, /football/germany/2-bundesliga/, /football/lithuania/i-lyga/, /football/mexico/liga-de-expansion-mx/</t>
   </si>
 </sst>
 </file>
@@ -9870,6 +9876,47 @@
         <v>367</v>
       </c>
     </row>
+    <row r="207">
+      <c r="A207" s="1" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B207" t="s">
+        <v>368</v>
+      </c>
+      <c r="C207" t="s">
+        <v>31</v>
+      </c>
+      <c r="D207" t="n">
+        <v>179.676146527131</v>
+      </c>
+      <c r="E207" t="n">
+        <v>40</v>
+      </c>
+      <c r="F207" t="n">
+        <v>1</v>
+      </c>
+      <c r="G207" t="n">
+        <v>245</v>
+      </c>
+      <c r="H207" t="n">
+        <v>67</v>
+      </c>
+      <c r="I207" t="n">
+        <v>178</v>
+      </c>
+      <c r="J207" t="n">
+        <v>14</v>
+      </c>
+      <c r="K207" t="n">
+        <v>3919</v>
+      </c>
+      <c r="L207" t="n">
+        <v>10</v>
+      </c>
+      <c r="M207" t="s">
+        <v>369</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-24]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="373">
   <si>
     <t>date</t>
   </si>
@@ -1131,6 +1131,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/colombia/primera-a/, /football/colombia/primera-b/, /football/estonia/meistriliiga/, /football/finland/ykkosliiga/, /football/paraguay/copa-de-primera/, /football/turkey/super-lig/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5e617748df235e0762e09974efc3903bd7087045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/colombia/primera-a/, /football/croatia/hnl/, /football/iceland/division-1/, /football/peru/liga-2/, /football/turkey/super-lig/</t>
   </si>
 </sst>
 </file>
@@ -9964,6 +9970,47 @@
         <v>371</v>
       </c>
     </row>
+    <row r="209">
+      <c r="A209" s="1" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B209" t="s">
+        <v>372</v>
+      </c>
+      <c r="C209" t="s">
+        <v>31</v>
+      </c>
+      <c r="D209" t="n">
+        <v>168.703181711833</v>
+      </c>
+      <c r="E209" t="n">
+        <v>48</v>
+      </c>
+      <c r="F209" t="n">
+        <v>1</v>
+      </c>
+      <c r="G209" t="n">
+        <v>312</v>
+      </c>
+      <c r="H209" t="n">
+        <v>98</v>
+      </c>
+      <c r="I209" t="n">
+        <v>214</v>
+      </c>
+      <c r="J209" t="n">
+        <v>8</v>
+      </c>
+      <c r="K209" t="n">
+        <v>4526</v>
+      </c>
+      <c r="L209" t="n">
+        <v>21</v>
+      </c>
+      <c r="M209" t="s">
+        <v>373</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-25]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="375">
   <si>
     <t>date</t>
   </si>
@@ -1137,6 +1137,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/colombia/primera-a/, /football/croatia/hnl/, /football/iceland/division-1/, /football/peru/liga-2/, /football/turkey/super-lig/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5a3271c28d1bf573f3abc0671a3ef337816cc84d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/ecuador/serie-b/, /football/estonia/meistriliiga/, /football/iceland/division-1/, /football/ireland/premier-division/, /football/ireland/division-1/, /football/lithuania/i-lyga/, /football/romania/superliga/</t>
   </si>
 </sst>
 </file>
@@ -10011,6 +10017,47 @@
         <v>373</v>
       </c>
     </row>
+    <row r="210">
+      <c r="A210" s="1" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B210" t="s">
+        <v>374</v>
+      </c>
+      <c r="C210" t="s">
+        <v>31</v>
+      </c>
+      <c r="D210" t="n">
+        <v>172.990753614903</v>
+      </c>
+      <c r="E210" t="n">
+        <v>57</v>
+      </c>
+      <c r="F210" t="n">
+        <v>1</v>
+      </c>
+      <c r="G210" t="n">
+        <v>335</v>
+      </c>
+      <c r="H210" t="n">
+        <v>129</v>
+      </c>
+      <c r="I210" t="n">
+        <v>206</v>
+      </c>
+      <c r="J210" t="n">
+        <v>19</v>
+      </c>
+      <c r="K210" t="n">
+        <v>4926</v>
+      </c>
+      <c r="L210" t="n">
+        <v>26</v>
+      </c>
+      <c r="M210" t="s">
+        <v>375</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-26]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="379">
   <si>
     <t>date</t>
   </si>
@@ -1149,6 +1149,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/bulgaria/vtora-liga/, /football/croatia/hnl/, /football/denmark/1st-division/, /football/finland/ykkosliiga/, /football/iceland/division-1/, /football/lithuania/i-lyga/, /football/malawi/super-league/, /football/paraguay/division-intermedia/, /football/peru/liga-1/, /football/poland/ekstraklasa/, /football/south-korea/k-league-2/, /football/turkey/super-lig/, /football/venezuela/liga-futve-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5a0e21ba89f4f88f1d8572abd4cc4b830e1624b2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/australia/npl-northern-nsw/, /football/austria/2-liga/, /football/denmark/1st-division/, /football/ecuador/serie-b/, /football/finland/ykkosliiga/, /football/paraguay/division-intermedia/, /football/peru/liga-1/, /football/poland/ekstraklasa/, /football/romania/superliga/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -10105,6 +10111,47 @@
         <v>377</v>
       </c>
     </row>
+    <row r="212">
+      <c r="A212" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B212" t="s">
+        <v>378</v>
+      </c>
+      <c r="C212" t="s">
+        <v>31</v>
+      </c>
+      <c r="D212" t="n">
+        <v>242.320657483737</v>
+      </c>
+      <c r="E212" t="n">
+        <v>54</v>
+      </c>
+      <c r="F212" t="n">
+        <v>1</v>
+      </c>
+      <c r="G212" t="n">
+        <v>293</v>
+      </c>
+      <c r="H212" t="n">
+        <v>74</v>
+      </c>
+      <c r="I212" t="n">
+        <v>219</v>
+      </c>
+      <c r="J212" t="n">
+        <v>42</v>
+      </c>
+      <c r="K212" t="n">
+        <v>5728</v>
+      </c>
+      <c r="L212" t="n">
+        <v>16</v>
+      </c>
+      <c r="M212" t="s">
+        <v>379</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-27]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="383">
   <si>
     <t>date</t>
   </si>
@@ -1161,6 +1161,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/colombia/primera-a/, /football/croatia/hnl/, /football/denmark/1st-division/, /football/finland/veikkausliiga/, /football/ireland/premier-division/, /football/lithuania/i-lyga/, /football/norway/obos-ligaen/, /football/norway/obos-ligaen/, /football/peru/liga-1/, /football/portugal/liga-portugal/, /football/slovenia/prva-liga/, /football/south-korea/k-league-2/, /football/turkey/super-lig/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6fd7e4f606d34580e3ea7ab3d79c5200b74098a9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/bulgaria/vtora-liga/, /football/ecuador/serie-b/, /football/estonia/meistriliiga/, /football/iceland/division-1/, /football/ireland/division-1/, /football/kazakhstan/premier-league/, /football/mexico/liga-de-expansion-mx/, /football/peru/liga-1/, /football/poland/ekstraklasa/, /football/slovenia/prva-liga/</t>
   </si>
 </sst>
 </file>
@@ -10199,6 +10205,47 @@
         <v>381</v>
       </c>
     </row>
+    <row r="214">
+      <c r="A214" s="1" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B214" t="s">
+        <v>382</v>
+      </c>
+      <c r="C214" t="s">
+        <v>31</v>
+      </c>
+      <c r="D214" t="n">
+        <v>246.898457364241</v>
+      </c>
+      <c r="E214" t="n">
+        <v>41</v>
+      </c>
+      <c r="F214" t="n">
+        <v>1</v>
+      </c>
+      <c r="G214" t="n">
+        <v>222</v>
+      </c>
+      <c r="H214" t="n">
+        <v>107</v>
+      </c>
+      <c r="I214" t="n">
+        <v>115</v>
+      </c>
+      <c r="J214" t="n">
+        <v>37</v>
+      </c>
+      <c r="K214" t="n">
+        <v>4523</v>
+      </c>
+      <c r="L214" t="n">
+        <v>13</v>
+      </c>
+      <c r="M214" t="s">
+        <v>383</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-28]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="385">
   <si>
     <t>date</t>
   </si>
@@ -1167,6 +1167,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/bulgaria/vtora-liga/, /football/ecuador/serie-b/, /football/estonia/meistriliiga/, /football/iceland/division-1/, /football/ireland/division-1/, /football/kazakhstan/premier-league/, /football/mexico/liga-de-expansion-mx/, /football/peru/liga-1/, /football/poland/ekstraklasa/, /football/slovenia/prva-liga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aa3f7537a321dbcbe2fdd26542abc179647f7832</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/kazakhstan/premier-league/, /football/lithuania/i-lyga/, /football/peru/liga-1/, /football/romania/superliga/, /football/slovenia/prva-liga/, /football/turkey/super-lig/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -10246,6 +10252,47 @@
         <v>383</v>
       </c>
     </row>
+    <row r="215">
+      <c r="A215" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B215" t="s">
+        <v>384</v>
+      </c>
+      <c r="C215" t="s">
+        <v>31</v>
+      </c>
+      <c r="D215" t="n">
+        <v>250.872381957372</v>
+      </c>
+      <c r="E215" t="n">
+        <v>38</v>
+      </c>
+      <c r="F215" t="n">
+        <v>1</v>
+      </c>
+      <c r="G215" t="n">
+        <v>277</v>
+      </c>
+      <c r="H215" t="n">
+        <v>86</v>
+      </c>
+      <c r="I215" t="n">
+        <v>191</v>
+      </c>
+      <c r="J215" t="n">
+        <v>22</v>
+      </c>
+      <c r="K215" t="n">
+        <v>4431</v>
+      </c>
+      <c r="L215" t="n">
+        <v>11</v>
+      </c>
+      <c r="M215" t="s">
+        <v>385</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-29]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="389">
   <si>
     <t>date</t>
   </si>
@@ -1179,6 +1179,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/australia/npl-act/, /football/canada/canadian-premier-league/, /football/colombia/primera-a/, /football/estonia/meistriliiga/, /football/ireland/division-1/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/slovenia/prva-liga/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a9b86c8aff597a362661f4e30e6865ed9dcdb850</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/australia/npl-act/, /football/belarus/vysshaya-liga/, /football/bulgaria/vtora-liga/, /football/canada/canadian-premier-league/, /football/chile/liga-de-primera/, /football/mexico/liga-de-expansion-mx/, /football/poland/division-1/, /football/slovenia/prva-liga/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -10340,6 +10346,47 @@
         <v>387</v>
       </c>
     </row>
+    <row r="217">
+      <c r="A217" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B217" t="s">
+        <v>388</v>
+      </c>
+      <c r="C217" t="s">
+        <v>31</v>
+      </c>
+      <c r="D217" t="n">
+        <v>236.005046149095</v>
+      </c>
+      <c r="E217" t="n">
+        <v>49</v>
+      </c>
+      <c r="F217" t="n">
+        <v>1</v>
+      </c>
+      <c r="G217" t="n">
+        <v>310</v>
+      </c>
+      <c r="H217" t="n">
+        <v>82</v>
+      </c>
+      <c r="I217" t="n">
+        <v>228</v>
+      </c>
+      <c r="J217" t="n">
+        <v>3</v>
+      </c>
+      <c r="K217" t="n">
+        <v>5018</v>
+      </c>
+      <c r="L217" t="n">
+        <v>19</v>
+      </c>
+      <c r="M217" t="s">
+        <v>389</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-30]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="393">
   <si>
     <t>date</t>
   </si>
@@ -1191,6 +1191,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/kazakhstan/premier-league/, /football/peru/liga-1/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/, /football/venezuela/liga-futve-2/, /football/venezuela/liga-futve-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5c9f7359af25ec55c0cf912425e438d62be49d1e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/bulgaria/vtora-liga/, /football/canada/canadian-premier-league/, /football/chile/liga-de-ascenso/, /football/estonia/esiliiga/, /football/faroe-islands/premier-league/, /football/peru/liga-1/, /football/turkey/super-lig/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -10434,6 +10440,47 @@
         <v>391</v>
       </c>
     </row>
+    <row r="219">
+      <c r="A219" s="1" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B219" t="s">
+        <v>392</v>
+      </c>
+      <c r="C219" t="s">
+        <v>31</v>
+      </c>
+      <c r="D219" t="n">
+        <v>279.775796906153</v>
+      </c>
+      <c r="E219" t="n">
+        <v>48</v>
+      </c>
+      <c r="F219" t="n">
+        <v>0</v>
+      </c>
+      <c r="G219" t="n">
+        <v>293</v>
+      </c>
+      <c r="H219" t="n">
+        <v>66</v>
+      </c>
+      <c r="I219" t="n">
+        <v>227</v>
+      </c>
+      <c r="J219" t="n">
+        <v>9</v>
+      </c>
+      <c r="K219" t="n">
+        <v>5014</v>
+      </c>
+      <c r="L219" t="n">
+        <v>17</v>
+      </c>
+      <c r="M219" t="s">
+        <v>393</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-07-31]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="397">
   <si>
     <t>date</t>
   </si>
@@ -1203,6 +1203,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/chile/liga-de-ascenso/, /football/paraguay/copa-de-primera/, /football/paraguay/division-intermedia/, /football/turkey/super-lig/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">063404c8de5197c870d9cbba1824a9773a5c74aa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/canada/canadian-premier-league/, /football/faroe-islands/premier-league/, /football/latvia/nakotnes-liga/, /football/lithuania/i-lyga/, /football/paraguay/division-intermedia/, /football/south-america/copa-sudamericana/, /football/south-america/copa-sudamericana/</t>
   </si>
 </sst>
 </file>
@@ -10528,6 +10534,47 @@
         <v>395</v>
       </c>
     </row>
+    <row r="221">
+      <c r="A221" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B221" t="s">
+        <v>396</v>
+      </c>
+      <c r="C221" t="s">
+        <v>31</v>
+      </c>
+      <c r="D221" t="n">
+        <v>231.983023118973</v>
+      </c>
+      <c r="E221" t="n">
+        <v>58</v>
+      </c>
+      <c r="F221" t="n">
+        <v>1</v>
+      </c>
+      <c r="G221" t="n">
+        <v>348</v>
+      </c>
+      <c r="H221" t="n">
+        <v>122</v>
+      </c>
+      <c r="I221" t="n">
+        <v>226</v>
+      </c>
+      <c r="J221" t="n">
+        <v>6</v>
+      </c>
+      <c r="K221" t="n">
+        <v>5405</v>
+      </c>
+      <c r="L221" t="n">
+        <v>24</v>
+      </c>
+      <c r="M221" t="s">
+        <v>397</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-01]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="399">
   <si>
     <t>date</t>
   </si>
@@ -1209,6 +1209,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/canada/canadian-premier-league/, /football/faroe-islands/premier-league/, /football/latvia/nakotnes-liga/, /football/lithuania/i-lyga/, /football/paraguay/division-intermedia/, /football/south-america/copa-sudamericana/, /football/south-america/copa-sudamericana/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">331752795fb354b50de0fcae8344badb49543f37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/australia/npl-act/, /football/bulgaria/vtora-liga/, /football/canada/canadian-premier-league/, /football/chile/liga-de-primera/, /football/colombia/primera-a/, /football/moldova/super-liga/, /football/romania/superliga/, /football/romania/liga-2/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -10575,6 +10581,47 @@
         <v>397</v>
       </c>
     </row>
+    <row r="222">
+      <c r="A222" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B222" t="s">
+        <v>398</v>
+      </c>
+      <c r="C222" t="s">
+        <v>31</v>
+      </c>
+      <c r="D222" t="n">
+        <v>289.418463623524</v>
+      </c>
+      <c r="E222" t="n">
+        <v>69</v>
+      </c>
+      <c r="F222" t="n">
+        <v>0</v>
+      </c>
+      <c r="G222" t="n">
+        <v>371</v>
+      </c>
+      <c r="H222" t="n">
+        <v>154</v>
+      </c>
+      <c r="I222" t="n">
+        <v>217</v>
+      </c>
+      <c r="J222" t="n">
+        <v>26</v>
+      </c>
+      <c r="K222" t="n">
+        <v>6381</v>
+      </c>
+      <c r="L222" t="n">
+        <v>32</v>
+      </c>
+      <c r="M222" t="s">
+        <v>399</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-02]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="403">
   <si>
     <t>date</t>
   </si>
@@ -1221,6 +1221,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/esiliiga/, /football/finland/ykkosliiga/, /football/lithuania/i-lyga/, /football/moldova/super-liga/, /football/poland/ekstraklasa/, /football/turkey/super-lig/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">be63741559619e74fe50c7c9140e2b4d0c0d6710</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/northern-ireland/nifl-premiership/, /football/romania/superliga/, /football/sweden/superettan/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -10669,6 +10675,47 @@
         <v>401</v>
       </c>
     </row>
+    <row r="224">
+      <c r="A224" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B224" t="s">
+        <v>402</v>
+      </c>
+      <c r="C224" t="s">
+        <v>31</v>
+      </c>
+      <c r="D224" t="n">
+        <v>248.826921586196</v>
+      </c>
+      <c r="E224" t="n">
+        <v>68</v>
+      </c>
+      <c r="F224" t="n">
+        <v>0</v>
+      </c>
+      <c r="G224" t="n">
+        <v>307</v>
+      </c>
+      <c r="H224" t="n">
+        <v>92</v>
+      </c>
+      <c r="I224" t="n">
+        <v>215</v>
+      </c>
+      <c r="J224" t="n">
+        <v>50</v>
+      </c>
+      <c r="K224" t="n">
+        <v>6202</v>
+      </c>
+      <c r="L224" t="n">
+        <v>24</v>
+      </c>
+      <c r="M224" t="s">
+        <v>403</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-03]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="407">
   <si>
     <t>date</t>
   </si>
@@ -1233,6 +1233,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/2-liga/, /football/bulgaria/vtora-liga/, /football/estonia/meistriliiga/, /football/lithuania/i-lyga/, /football/moldova/super-liga/, /football/peru/liga-1/, /football/poland/ekstraklasa/, /football/poland/division-1/, /football/romania/superliga/, /football/slovenia/prva-liga/, /football/south-korea/k-league-2/, /football/sweden/superettan/, /football/turkey/super-lig/, /football/usa/usl-championship/, /football/venezuela/liga-futve-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">43ad8122816532b5ad46e512d7ea540c156a1fe2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/croatia/hnl/, /football/estonia/meistriliiga/, /football/iceland/division-1/, /football/mexico/liga-de-expansion-mx/, /football/poland/ekstraklasa/, /football/poland/division-1/, /football/romania/superliga/</t>
   </si>
 </sst>
 </file>
@@ -10763,6 +10769,47 @@
         <v>405</v>
       </c>
     </row>
+    <row r="226">
+      <c r="A226" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B226" t="s">
+        <v>406</v>
+      </c>
+      <c r="C226" t="s">
+        <v>31</v>
+      </c>
+      <c r="D226" t="n">
+        <v>302.01491830349</v>
+      </c>
+      <c r="E226" t="n">
+        <v>57</v>
+      </c>
+      <c r="F226" t="n">
+        <v>0</v>
+      </c>
+      <c r="G226" t="n">
+        <v>328</v>
+      </c>
+      <c r="H226" t="n">
+        <v>117</v>
+      </c>
+      <c r="I226" t="n">
+        <v>211</v>
+      </c>
+      <c r="J226" t="n">
+        <v>46</v>
+      </c>
+      <c r="K226" t="n">
+        <v>5945</v>
+      </c>
+      <c r="L226" t="n">
+        <v>26</v>
+      </c>
+      <c r="M226" t="s">
+        <v>407</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-04]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="411">
   <si>
     <t>date</t>
   </si>
@@ -1245,6 +1245,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/croatia/hnl/, /football/estonia/meistriliiga/, /football/peru/liga-1/, /football/poland/division-1/, /football/romania/superliga/, /football/slovenia/prva-liga/, /football/slovenia/prva-liga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0deb675b9884203c10baaf2cc9e472b00204595c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/colombia/primera-a/, /football/croatia/hnl/, /football/iceland/division-1/, /football/ireland/division-1/, /football/kazakhstan/premier-league/, /football/mexico/liga-de-expansion-mx/, /football/mexico/liga-de-expansion-mx/, /football/peru/liga-1/, /football/poland/ekstraklasa/, /football/poland/division-1/, /football/romania/superliga/, /football/turkey/1-lig/</t>
   </si>
 </sst>
 </file>
@@ -10857,6 +10863,47 @@
         <v>409</v>
       </c>
     </row>
+    <row r="228">
+      <c r="A228" s="1" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B228" t="s">
+        <v>410</v>
+      </c>
+      <c r="C228" t="s">
+        <v>31</v>
+      </c>
+      <c r="D228" t="n">
+        <v>315.35932239294</v>
+      </c>
+      <c r="E228" t="n">
+        <v>47</v>
+      </c>
+      <c r="F228" t="n">
+        <v>0</v>
+      </c>
+      <c r="G228" t="n">
+        <v>341</v>
+      </c>
+      <c r="H228" t="n">
+        <v>123</v>
+      </c>
+      <c r="I228" t="n">
+        <v>218</v>
+      </c>
+      <c r="J228" t="n">
+        <v>9</v>
+      </c>
+      <c r="K228" t="n">
+        <v>5770</v>
+      </c>
+      <c r="L228" t="n">
+        <v>15</v>
+      </c>
+      <c r="M228" t="s">
+        <v>411</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-05]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="415">
   <si>
     <t>date</t>
   </si>
@@ -1257,6 +1257,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belgium/jupiler-pro-league/, /football/finland/ykkosliiga/, /football/iceland/division-1/, /football/ireland/premier-division/, /football/kazakhstan/premier-league/, /football/mexico/liga-de-expansion-mx/, /football/peru/liga-1/, /football/peru/liga-1/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">856c472455cf7a0b3e14873489589e1990b71479</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/australia/npl-northern-nsw/, /football/austria/2-liga/, /football/bulgaria/vtora-liga/, /football/iceland/division-1/, /football/kazakhstan/premier-league/, /football/slovenia/prva-liga/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -10951,6 +10957,47 @@
         <v>413</v>
       </c>
     </row>
+    <row r="230">
+      <c r="A230" s="1" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B230" t="s">
+        <v>414</v>
+      </c>
+      <c r="C230" t="s">
+        <v>31</v>
+      </c>
+      <c r="D230" t="n">
+        <v>186.596321205298</v>
+      </c>
+      <c r="E230" t="n">
+        <v>59</v>
+      </c>
+      <c r="F230" t="n">
+        <v>0</v>
+      </c>
+      <c r="G230" t="n">
+        <v>416</v>
+      </c>
+      <c r="H230" t="n">
+        <v>143</v>
+      </c>
+      <c r="I230" t="n">
+        <v>273</v>
+      </c>
+      <c r="J230" t="n">
+        <v>8</v>
+      </c>
+      <c r="K230" t="n">
+        <v>6475</v>
+      </c>
+      <c r="L230" t="n">
+        <v>26</v>
+      </c>
+      <c r="M230" t="s">
+        <v>415</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-07]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="419">
   <si>
     <t>date</t>
   </si>
@@ -1269,6 +1269,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/pershaya-liga/, /football/estonia/esiliiga/, /football/iceland/division-1/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/northern-ireland/nifl-premiership/, /football/paraguay/copa-de-primera/, /football/peru/liga-1/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6fbc198e0a31b4db8bc05086c8a9aa5082c8c36b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/faroe-islands/premier-league/, /football/romania/superliga/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -11045,6 +11051,47 @@
         <v>417</v>
       </c>
     </row>
+    <row r="232">
+      <c r="A232" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B232" t="s">
+        <v>418</v>
+      </c>
+      <c r="C232" t="s">
+        <v>31</v>
+      </c>
+      <c r="D232" t="n">
+        <v>248.807817363739</v>
+      </c>
+      <c r="E232" t="n">
+        <v>76</v>
+      </c>
+      <c r="F232" t="n">
+        <v>1</v>
+      </c>
+      <c r="G232" t="n">
+        <v>518</v>
+      </c>
+      <c r="H232" t="n">
+        <v>212</v>
+      </c>
+      <c r="I232" t="n">
+        <v>306</v>
+      </c>
+      <c r="J232" t="n">
+        <v>13</v>
+      </c>
+      <c r="K232" t="n">
+        <v>7292</v>
+      </c>
+      <c r="L232" t="n">
+        <v>33</v>
+      </c>
+      <c r="M232" t="s">
+        <v>419</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-08]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="423">
   <si>
     <t>date</t>
   </si>
@@ -1281,6 +1281,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/armenia/premier-league/, /football/latvia/nakotnes-liga/, /football/lithuania/i-lyga/, /football/peru/liga-1/, /football/romania/superliga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e08e9a07a80306948bd064e18d69aa95c257d2c7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/romania/superliga/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -11139,6 +11145,47 @@
         <v>421</v>
       </c>
     </row>
+    <row r="234">
+      <c r="A234" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B234" t="s">
+        <v>422</v>
+      </c>
+      <c r="C234" t="s">
+        <v>31</v>
+      </c>
+      <c r="D234" t="n">
+        <v>266.904180081685</v>
+      </c>
+      <c r="E234" t="n">
+        <v>79</v>
+      </c>
+      <c r="F234" t="n">
+        <v>0</v>
+      </c>
+      <c r="G234" t="n">
+        <v>502</v>
+      </c>
+      <c r="H234" t="n">
+        <v>186</v>
+      </c>
+      <c r="I234" t="n">
+        <v>316</v>
+      </c>
+      <c r="J234" t="n">
+        <v>25</v>
+      </c>
+      <c r="K234" t="n">
+        <v>7389</v>
+      </c>
+      <c r="L234" t="n">
+        <v>34</v>
+      </c>
+      <c r="M234" t="s">
+        <v>423</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-09]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="427">
   <si>
     <t>date</t>
   </si>
@@ -1293,6 +1293,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/bundesliga/, /football/austria/2-liga/, /football/bulgaria/vtora-liga/, /football/bulgaria/vtora-liga/, /football/costa-rica/liga-de-ascenso/, /football/northern-ireland/nifl-premiership/, /football/romania/superliga/, /football/slovakia/nike-liga/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">44e4b2481a1cf0fa8c108f35f9b60ac0cd64b412</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/bundesliga/, /football/denmark/1st-division/, /football/france/ligue-2/, /football/france/ligue-2/, /football/france/ligue-2/, /football/latvia/virsliga/, /football/northern-ireland/nifl-premiership/, /football/peru/liga-1/, /football/south-korea/k-league-2/, /football/sweden/superettan/</t>
   </si>
 </sst>
 </file>
@@ -11233,6 +11239,47 @@
         <v>425</v>
       </c>
     </row>
+    <row r="236">
+      <c r="A236" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B236" t="s">
+        <v>426</v>
+      </c>
+      <c r="C236" t="s">
+        <v>31</v>
+      </c>
+      <c r="D236" t="n">
+        <v>282.536425383886</v>
+      </c>
+      <c r="E236" t="n">
+        <v>77</v>
+      </c>
+      <c r="F236" t="n">
+        <v>0</v>
+      </c>
+      <c r="G236" t="n">
+        <v>394</v>
+      </c>
+      <c r="H236" t="n">
+        <v>79</v>
+      </c>
+      <c r="I236" t="n">
+        <v>315</v>
+      </c>
+      <c r="J236" t="n">
+        <v>37</v>
+      </c>
+      <c r="K236" t="n">
+        <v>7525</v>
+      </c>
+      <c r="L236" t="n">
+        <v>27</v>
+      </c>
+      <c r="M236" t="s">
+        <v>427</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-10]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="429">
   <si>
     <t>date</t>
   </si>
@@ -1299,6 +1299,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/bundesliga/, /football/denmark/1st-division/, /football/france/ligue-2/, /football/france/ligue-2/, /football/france/ligue-2/, /football/latvia/virsliga/, /football/northern-ireland/nifl-premiership/, /football/peru/liga-1/, /football/south-korea/k-league-2/, /football/sweden/superettan/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8670ddfccd44fd47283a608aa65b93d56350c10f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/finland/veikkausliiga/, /football/france/ligue-2/, /football/northern-ireland/nifl-premiership/, /football/norway/obos-ligaen/, /football/peru/liga-1/, /football/poland/division-1/, /football/slovenia/prva-liga/, /football/sweden/superettan/</t>
   </si>
 </sst>
 </file>
@@ -11280,6 +11286,47 @@
         <v>427</v>
       </c>
     </row>
+    <row r="237">
+      <c r="A237" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B237" t="s">
+        <v>428</v>
+      </c>
+      <c r="C237" t="s">
+        <v>31</v>
+      </c>
+      <c r="D237" t="n">
+        <v>239.035535009702</v>
+      </c>
+      <c r="E237" t="n">
+        <v>57</v>
+      </c>
+      <c r="F237" t="n">
+        <v>0</v>
+      </c>
+      <c r="G237" t="n">
+        <v>331</v>
+      </c>
+      <c r="H237" t="n">
+        <v>97</v>
+      </c>
+      <c r="I237" t="n">
+        <v>234</v>
+      </c>
+      <c r="J237" t="n">
+        <v>146</v>
+      </c>
+      <c r="K237" t="n">
+        <v>6759</v>
+      </c>
+      <c r="L237" t="n">
+        <v>12</v>
+      </c>
+      <c r="M237" t="s">
+        <v>429</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-11]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="433">
   <si>
     <t>date</t>
   </si>
@@ -1311,6 +1311,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/2-liga/, /football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/estonia/meistriliiga/, /football/france/ligue-2/, /football/kazakhstan/premier-league/, /football/netherlands/eerste-divisie/, /football/paraguay/copa-de-primera/, /football/peru/liga-1/, /football/poland/division-1/, /football/poland/division-1/, /football/slovenia/prva-liga/, /football/slovenia/prva-liga/, /football/slovenia/prva-liga/, /football/turkey/1-lig/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9bdd3da1538f0a679e5825c2193f3ba5a9d21897</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/colombia/primera-a/, /football/estonia/meistriliiga/, /football/france/ligue-2/, /football/honduras/liga-nacional/, /football/iceland/division-1/, /football/kazakhstan/premier-league/, /football/northern-ireland/nifl-premiership/, /football/peru/liga-1/, /football/slovenia/prva-liga/</t>
   </si>
 </sst>
 </file>
@@ -11374,6 +11380,47 @@
         <v>431</v>
       </c>
     </row>
+    <row r="239">
+      <c r="A239" s="1" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B239" t="s">
+        <v>432</v>
+      </c>
+      <c r="C239" t="s">
+        <v>31</v>
+      </c>
+      <c r="D239" t="n">
+        <v>223.644102605184</v>
+      </c>
+      <c r="E239" t="n">
+        <v>52</v>
+      </c>
+      <c r="F239" t="n">
+        <v>0</v>
+      </c>
+      <c r="G239" t="n">
+        <v>378</v>
+      </c>
+      <c r="H239" t="n">
+        <v>109</v>
+      </c>
+      <c r="I239" t="n">
+        <v>269</v>
+      </c>
+      <c r="J239" t="n">
+        <v>14</v>
+      </c>
+      <c r="K239" t="n">
+        <v>6579</v>
+      </c>
+      <c r="L239" t="n">
+        <v>19</v>
+      </c>
+      <c r="M239" t="s">
+        <v>433</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-12]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="437">
   <si>
     <t>date</t>
   </si>
@@ -1323,6 +1323,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/belgium/jupiler-pro-league/, /football/finland/ykkosliiga/, /football/honduras/liga-nacional/, /football/lithuania/i-lyga/, /football/northern-ireland/nifl-premiership/, /football/paraguay/copa-de-primera/, /football/peru/liga-1/, /football/turkey/1-lig/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09a29cc77fbafc6d075ecec553263e1084a692ec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/estonia/meistriliiga/, /football/france/ligue-2/, /football/honduras/liga-nacional/, /football/kazakhstan/premier-league/, /football/lithuania/i-lyga/, /football/mexico/liga-de-expansion-mx/, /football/peru/liga-1/, /football/poland/ekstraklasa/, /football/turkey/1-lig/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -11468,6 +11474,47 @@
         <v>435</v>
       </c>
     </row>
+    <row r="241">
+      <c r="A241" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B241" t="s">
+        <v>436</v>
+      </c>
+      <c r="C241" t="s">
+        <v>31</v>
+      </c>
+      <c r="D241" t="n">
+        <v>258.721691075961</v>
+      </c>
+      <c r="E241" t="n">
+        <v>50</v>
+      </c>
+      <c r="F241" t="n">
+        <v>0</v>
+      </c>
+      <c r="G241" t="n">
+        <v>346</v>
+      </c>
+      <c r="H241" t="n">
+        <v>119</v>
+      </c>
+      <c r="I241" t="n">
+        <v>227</v>
+      </c>
+      <c r="J241" t="n">
+        <v>4</v>
+      </c>
+      <c r="K241" t="n">
+        <v>6054</v>
+      </c>
+      <c r="L241" t="n">
+        <v>19</v>
+      </c>
+      <c r="M241" t="s">
+        <v>437</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-13]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="441">
   <si>
     <t>date</t>
   </si>
@@ -1335,6 +1335,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/canada/canadian-premier-league/, /football/france/ligue-2/, /football/lithuania/i-lyga/, /football/paraguay/copa-de-primera/, /football/peru/liga-1/, /football/romania/liga-2/, /football/turkey/1-lig/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">980e680c80b62e3a2a33a770945cf7bcb0fbd837</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/chile/liga-de-ascenso/, /football/finland/ykkosliiga/, /football/kazakhstan/premier-league/, /football/kazakhstan/premier-league/, /football/lithuania/i-lyga/, /football/northern-ireland/nifl-premiership/, /football/norway/eliteserien/, /football/paraguay/copa-de-primera/, /football/peru/liga-1/, /football/turkey/1-lig/</t>
   </si>
 </sst>
 </file>
@@ -11562,6 +11568,47 @@
         <v>439</v>
       </c>
     </row>
+    <row r="243">
+      <c r="A243" s="1" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B243" t="s">
+        <v>440</v>
+      </c>
+      <c r="C243" t="s">
+        <v>31</v>
+      </c>
+      <c r="D243" t="n">
+        <v>290.512652738889</v>
+      </c>
+      <c r="E243" t="n">
+        <v>61</v>
+      </c>
+      <c r="F243" t="n">
+        <v>0</v>
+      </c>
+      <c r="G243" t="n">
+        <v>443</v>
+      </c>
+      <c r="H243" t="n">
+        <v>159</v>
+      </c>
+      <c r="I243" t="n">
+        <v>284</v>
+      </c>
+      <c r="J243" t="n">
+        <v>6</v>
+      </c>
+      <c r="K243" t="n">
+        <v>6746</v>
+      </c>
+      <c r="L243" t="n">
+        <v>22</v>
+      </c>
+      <c r="M243" t="s">
+        <v>441</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-14]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="445">
   <si>
     <t>date</t>
   </si>
@@ -1347,6 +1347,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/el-salvador/primera-division/, /football/kazakhstan/premier-league/, /football/paraguay/copa-de-primera/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2439bc045073ba419fde407bae51dadf94b721ae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/colombia/primera-a/, /football/colombia/primera-b/, /football/england/premier-league/, /football/estonia/esiliiga/, /football/faroe-islands/premier-league/, /football/paraguay/division-intermedia/, /football/peru/liga-1/</t>
   </si>
 </sst>
 </file>
@@ -11656,6 +11662,47 @@
         <v>443</v>
       </c>
     </row>
+    <row r="245">
+      <c r="A245" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B245" t="s">
+        <v>444</v>
+      </c>
+      <c r="C245" t="s">
+        <v>31</v>
+      </c>
+      <c r="D245" t="n">
+        <v>294.148890785376</v>
+      </c>
+      <c r="E245" t="n">
+        <v>76</v>
+      </c>
+      <c r="F245" t="n">
+        <v>0</v>
+      </c>
+      <c r="G245" t="n">
+        <v>534</v>
+      </c>
+      <c r="H245" t="n">
+        <v>211</v>
+      </c>
+      <c r="I245" t="n">
+        <v>323</v>
+      </c>
+      <c r="J245" t="n">
+        <v>6</v>
+      </c>
+      <c r="K245" t="n">
+        <v>7865</v>
+      </c>
+      <c r="L245" t="n">
+        <v>37</v>
+      </c>
+      <c r="M245" t="s">
+        <v>445</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-15]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="447">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="449">
   <si>
     <t>date</t>
   </si>
@@ -1359,6 +1359,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/colombia/primera-a/, /football/fiji/premier-league/, /football/germany/2-bundesliga/, /football/greece/super-league/, /football/netherlands/eerste-divisie/, /football/peru/liga-1/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1107839d692e5cd4ebc48e2f20c44622c84b1aee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/pershaya-liga/, /football/bulgaria/vtora-liga/, /football/chile/liga-de-primera/, /football/china/super-league/, /football/colombia/primera-a/, /football/estonia/esiliiga/, /football/finland/ykkosliiga/, /football/iraq/stars-league/, /football/northern-ireland/nifl-premiership/, /football/peru/liga-1/, /football/romania/superliga/, /football/venezuela/liga-futve-2/</t>
   </si>
 </sst>
 </file>
@@ -11750,6 +11756,47 @@
         <v>447</v>
       </c>
     </row>
+    <row r="247">
+      <c r="A247" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B247" t="s">
+        <v>448</v>
+      </c>
+      <c r="C247" t="s">
+        <v>31</v>
+      </c>
+      <c r="D247" t="n">
+        <v>342.269139655431</v>
+      </c>
+      <c r="E247" t="n">
+        <v>73</v>
+      </c>
+      <c r="F247" t="n">
+        <v>0</v>
+      </c>
+      <c r="G247" t="n">
+        <v>399</v>
+      </c>
+      <c r="H247" t="n">
+        <v>172</v>
+      </c>
+      <c r="I247" t="n">
+        <v>227</v>
+      </c>
+      <c r="J247" t="n">
+        <v>103</v>
+      </c>
+      <c r="K247" t="n">
+        <v>7397</v>
+      </c>
+      <c r="L247" t="n">
+        <v>26</v>
+      </c>
+      <c r="M247" t="s">
+        <v>449</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-16]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="451">
   <si>
     <t>date</t>
   </si>
@@ -1365,6 +1365,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/pershaya-liga/, /football/bulgaria/vtora-liga/, /football/chile/liga-de-primera/, /football/china/super-league/, /football/colombia/primera-a/, /football/estonia/esiliiga/, /football/finland/ykkosliiga/, /football/iraq/stars-league/, /football/northern-ireland/nifl-premiership/, /football/peru/liga-1/, /football/romania/superliga/, /football/venezuela/liga-futve-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">33c20ed48c54d03ed6a29c2b3fbc69ec2bf8581c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/bosnia-and-herzegovina/prva-liga-fbih/, /football/chile/liga-de-primera/, /football/china/super-league/, /football/costa-rica/liga-de-ascenso/, /football/croatia/hnl/, /football/estonia/meistriliiga/, /football/finland/veikkausliiga/, /football/poland/division-1/, /football/portugal/liga-portugal-2/, /football/south-korea/k-league-2/, /football/sweden/superettan/, /football/turkey/1-lig/, /football/ukraine/premier-league/, /football/usa/usl-championship/, /football/venezuela/liga-futve/, /football/venezuela/liga-futve-2/</t>
   </si>
 </sst>
 </file>
@@ -11797,6 +11803,47 @@
         <v>449</v>
       </c>
     </row>
+    <row r="248">
+      <c r="A248" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B248" t="s">
+        <v>450</v>
+      </c>
+      <c r="C248" t="s">
+        <v>31</v>
+      </c>
+      <c r="D248" t="n">
+        <v>339.5805605491</v>
+      </c>
+      <c r="E248" t="n">
+        <v>69</v>
+      </c>
+      <c r="F248" t="n">
+        <v>0</v>
+      </c>
+      <c r="G248" t="n">
+        <v>479</v>
+      </c>
+      <c r="H248" t="n">
+        <v>110</v>
+      </c>
+      <c r="I248" t="n">
+        <v>369</v>
+      </c>
+      <c r="J248" t="n">
+        <v>119</v>
+      </c>
+      <c r="K248" t="n">
+        <v>8245</v>
+      </c>
+      <c r="L248" t="n">
+        <v>18</v>
+      </c>
+      <c r="M248" t="s">
+        <v>451</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-17]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="453">
   <si>
     <t>date</t>
   </si>
@@ -1371,6 +1371,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/2-liga/, /football/bosnia-and-herzegovina/prva-liga-fbih/, /football/chile/liga-de-primera/, /football/china/super-league/, /football/costa-rica/liga-de-ascenso/, /football/croatia/hnl/, /football/estonia/meistriliiga/, /football/finland/veikkausliiga/, /football/poland/division-1/, /football/portugal/liga-portugal-2/, /football/south-korea/k-league-2/, /football/sweden/superettan/, /football/turkey/1-lig/, /football/ukraine/premier-league/, /football/usa/usl-championship/, /football/venezuela/liga-futve/, /football/venezuela/liga-futve-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6ae72ad7c6f437f3c77f4a161bd6856adaf87ef2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/china/super-league/, /football/egypt/premier-league/, /football/latvia/virsliga/, /football/northern-ireland/nifl-premiership/, /football/portugal/liga-portugal-2/, /football/romania/superliga/, /football/south-korea/k-league-2/, /football/sweden/superettan/, /football/turkey/1-lig/, /football/ukraine/premier-league/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -11844,6 +11850,47 @@
         <v>451</v>
       </c>
     </row>
+    <row r="249">
+      <c r="A249" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B249" t="s">
+        <v>452</v>
+      </c>
+      <c r="C249" t="s">
+        <v>31</v>
+      </c>
+      <c r="D249" t="n">
+        <v>240.187648129463</v>
+      </c>
+      <c r="E249" t="n">
+        <v>48</v>
+      </c>
+      <c r="F249" t="n">
+        <v>0</v>
+      </c>
+      <c r="G249" t="n">
+        <v>285</v>
+      </c>
+      <c r="H249" t="n">
+        <v>74</v>
+      </c>
+      <c r="I249" t="n">
+        <v>211</v>
+      </c>
+      <c r="J249" t="n">
+        <v>62</v>
+      </c>
+      <c r="K249" t="n">
+        <v>5653</v>
+      </c>
+      <c r="L249" t="n">
+        <v>14</v>
+      </c>
+      <c r="M249" t="s">
+        <v>453</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-18]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="455">
   <si>
     <t>date</t>
   </si>
@@ -1377,6 +1377,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/china/super-league/, /football/egypt/premier-league/, /football/latvia/virsliga/, /football/northern-ireland/nifl-premiership/, /football/portugal/liga-portugal-2/, /football/romania/superliga/, /football/south-korea/k-league-2/, /football/sweden/superettan/, /football/turkey/1-lig/, /football/ukraine/premier-league/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">641da2d7df03642a6416f16e7f1e5945577eec19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/colombia/primera-b/, /football/iceland/division-1/, /football/ireland/division-1/, /football/kazakhstan/premier-league/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/northern-ireland/nifl-premiership/, /football/romania/liga-2/, /football/sweden/superettan/, /football/turkey/1-lig/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -11891,6 +11897,47 @@
         <v>453</v>
       </c>
     </row>
+    <row r="250">
+      <c r="A250" s="1" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B250" t="s">
+        <v>454</v>
+      </c>
+      <c r="C250" t="s">
+        <v>31</v>
+      </c>
+      <c r="D250" t="n">
+        <v>274.392261314392</v>
+      </c>
+      <c r="E250" t="n">
+        <v>56</v>
+      </c>
+      <c r="F250" t="n">
+        <v>1</v>
+      </c>
+      <c r="G250" t="n">
+        <v>407</v>
+      </c>
+      <c r="H250" t="n">
+        <v>185</v>
+      </c>
+      <c r="I250" t="n">
+        <v>222</v>
+      </c>
+      <c r="J250" t="n">
+        <v>27</v>
+      </c>
+      <c r="K250" t="n">
+        <v>6725</v>
+      </c>
+      <c r="L250" t="n">
+        <v>18</v>
+      </c>
+      <c r="M250" t="s">
+        <v>455</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-08-19]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="457">
   <si>
     <t>date</t>
   </si>
@@ -1383,6 +1383,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/colombia/primera-b/, /football/iceland/division-1/, /football/ireland/division-1/, /football/kazakhstan/premier-league/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/northern-ireland/nifl-premiership/, /football/romania/liga-2/, /football/sweden/superettan/, /football/turkey/1-lig/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bfe8407153c4400995449c91759fb6b03e6be9f5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/canada/canadian-premier-league/, /football/egypt/premier-league/, /football/el-salvador/primera-division/, /football/estonia/esiliiga/, /football/guatemala/liga-nacional/, /football/iceland/division-1/, /football/northern-ireland/nifl-premiership/, /football/paraguay/copa-de-primera/, /football/peru/liga-1/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -11938,6 +11944,47 @@
         <v>455</v>
       </c>
     </row>
+    <row r="251">
+      <c r="A251" s="1" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B251" t="s">
+        <v>456</v>
+      </c>
+      <c r="C251" t="s">
+        <v>31</v>
+      </c>
+      <c r="D251" t="n">
+        <v>265.079077374935</v>
+      </c>
+      <c r="E251" t="n">
+        <v>57</v>
+      </c>
+      <c r="F251" t="n">
+        <v>0</v>
+      </c>
+      <c r="G251" t="n">
+        <v>395</v>
+      </c>
+      <c r="H251" t="n">
+        <v>125</v>
+      </c>
+      <c r="I251" t="n">
+        <v>270</v>
+      </c>
+      <c r="J251" t="n">
+        <v>8</v>
+      </c>
+      <c r="K251" t="n">
+        <v>6791</v>
+      </c>
+      <c r="L251" t="n">
+        <v>20</v>
+      </c>
+      <c r="M251" t="s">
+        <v>457</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>